<commit_message>
Updated Gantt and Documentation to reflect current standing
</commit_message>
<xml_diff>
--- a/Gantt Zeitplan Josiah Spilker.xlsx
+++ b/Gantt Zeitplan Josiah Spilker.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1DA0B313-9E82-4B7E-BCAF-0F02F07A6644}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1D1EC714-81D8-4DD8-BE18-6DE63698BD93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43095" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="29010" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Project plan" sheetId="11" r:id="rId1"/>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="168">
   <si>
     <t>EINFACHES GANTT-DIAGRAMM von Vertex42.com</t>
   </si>
@@ -547,31 +547,34 @@
     <t>Wed.</t>
   </si>
   <si>
-    <t>T3 : Decide                                              5h</t>
-  </si>
-  <si>
-    <t>T5 : Control                                              6h</t>
-  </si>
-  <si>
-    <t>T1 : Inform                                               3h</t>
-  </si>
-  <si>
-    <t>T2 : Plan                                                 14h</t>
-  </si>
-  <si>
     <t>27.04.2026                                   / = &lt;1h</t>
   </si>
   <si>
-    <t>T0 : Documentation/Administration  16h</t>
-  </si>
-  <si>
-    <t>T4 : Realise                                            18h</t>
-  </si>
-  <si>
-    <t>T6 : Evaluate                                          8h</t>
-  </si>
-  <si>
     <t>T7 : Buffer                                             8h</t>
+  </si>
+  <si>
+    <t>T1 : Inform                                       3h</t>
+  </si>
+  <si>
+    <t>T0 : Documentation/Admin.        16h</t>
+  </si>
+  <si>
+    <t>T2 : Plan                                         14h</t>
+  </si>
+  <si>
+    <t>T3 : Decide                                       5h</t>
+  </si>
+  <si>
+    <t>T4 : Realise                                    18h</t>
+  </si>
+  <si>
+    <t>T5 : Control                                      6h</t>
+  </si>
+  <si>
+    <t>T6 : Evaluate                                    8h</t>
+  </si>
+  <si>
+    <t>T7 : Buffer                                        8h</t>
   </si>
 </sst>
 </file>
@@ -2152,7 +2155,7 @@
     <xf numFmtId="43" fontId="5" fillId="0" borderId="3" applyFont="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="5" fillId="0" borderId="3" applyFont="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="262">
+  <cellXfs count="265">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2691,6 +2694,48 @@
     <xf numFmtId="0" fontId="0" fillId="51" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="36" fillId="53" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="53" borderId="53" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="53" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="53" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="51" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="51" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="48" borderId="45" xfId="12" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="48" borderId="17" xfId="12" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="48" borderId="45" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="48" borderId="17" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="53" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="47" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="35" fillId="46" borderId="45" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -2700,6 +2745,12 @@
     <xf numFmtId="0" fontId="35" fillId="46" borderId="41" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="35" fillId="10" borderId="69" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="10" borderId="68" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="35" fillId="9" borderId="45" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -2709,12 +2760,6 @@
     <xf numFmtId="0" fontId="35" fillId="9" borderId="41" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="10" borderId="69" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="10" borderId="68" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="35" fillId="3" borderId="45" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -2727,6 +2772,15 @@
     <xf numFmtId="0" fontId="35" fillId="10" borderId="61" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="35" fillId="2" borderId="45" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="2" borderId="61" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="44" borderId="67" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="35" fillId="6" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2736,18 +2790,9 @@
     <xf numFmtId="49" fontId="35" fillId="6" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="2" borderId="45" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="35" fillId="2" borderId="17" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="2" borderId="61" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="44" borderId="67" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="5" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -2775,6 +2820,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="45" xfId="12" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="17" xfId="12" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="45" xfId="12" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -2799,12 +2850,6 @@
     <xf numFmtId="0" fontId="5" fillId="10" borderId="45" xfId="12" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="45" xfId="12" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="17" xfId="12" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="61" xfId="12" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -2889,41 +2934,8 @@
     <xf numFmtId="0" fontId="32" fillId="52" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="53" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="53" borderId="53" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="50" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="53" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="53" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="51" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="51" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="48" borderId="45" xfId="12" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="48" borderId="17" xfId="12" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="48" borderId="45" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="48" borderId="17" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="58">
@@ -3523,233 +3535,233 @@
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.85546875" customWidth="1"/>
-    <col min="2" max="13" width="2.7109375" hidden="1" customWidth="1"/>
-    <col min="14" max="41" width="2.7109375" customWidth="1"/>
+    <col min="2" max="17" width="2.7109375" hidden="1" customWidth="1"/>
+    <col min="18" max="41" width="2.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:59" ht="29.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="203" t="s">
+      <c r="A1" s="217" t="s">
         <v>93</v>
       </c>
-      <c r="B1" s="203"/>
-      <c r="C1" s="203"/>
-      <c r="D1" s="203"/>
-      <c r="E1" s="203"/>
-      <c r="F1" s="203"/>
-      <c r="G1" s="203"/>
-      <c r="H1" s="203"/>
-      <c r="I1" s="203"/>
-      <c r="J1" s="203"/>
-      <c r="K1" s="203"/>
-      <c r="L1" s="203"/>
-      <c r="M1" s="203"/>
-      <c r="N1" s="203"/>
-      <c r="O1" s="203"/>
-      <c r="P1" s="203"/>
-      <c r="Q1" s="203"/>
-      <c r="R1" s="203"/>
-      <c r="S1" s="203"/>
-      <c r="T1" s="203"/>
-      <c r="U1" s="203"/>
-      <c r="V1" s="203"/>
-      <c r="W1" s="203"/>
-      <c r="X1" s="203"/>
-      <c r="Y1" s="203"/>
-      <c r="Z1" s="203"/>
-      <c r="AA1" s="203"/>
-      <c r="AB1" s="203"/>
-      <c r="AC1" s="203"/>
-      <c r="AD1" s="203"/>
-      <c r="AE1" s="203"/>
-      <c r="AF1" s="203"/>
-      <c r="AG1" s="203"/>
-      <c r="AH1" s="203"/>
-      <c r="AI1" s="203"/>
-      <c r="AJ1" s="203"/>
-      <c r="AK1" s="203"/>
-      <c r="AL1" s="203"/>
-      <c r="AM1" s="203"/>
-      <c r="AN1" s="203"/>
-      <c r="AO1" s="203"/>
+      <c r="B1" s="217"/>
+      <c r="C1" s="217"/>
+      <c r="D1" s="217"/>
+      <c r="E1" s="217"/>
+      <c r="F1" s="217"/>
+      <c r="G1" s="217"/>
+      <c r="H1" s="217"/>
+      <c r="I1" s="217"/>
+      <c r="J1" s="217"/>
+      <c r="K1" s="217"/>
+      <c r="L1" s="217"/>
+      <c r="M1" s="217"/>
+      <c r="N1" s="217"/>
+      <c r="O1" s="217"/>
+      <c r="P1" s="217"/>
+      <c r="Q1" s="217"/>
+      <c r="R1" s="217"/>
+      <c r="S1" s="217"/>
+      <c r="T1" s="217"/>
+      <c r="U1" s="217"/>
+      <c r="V1" s="217"/>
+      <c r="W1" s="217"/>
+      <c r="X1" s="217"/>
+      <c r="Y1" s="217"/>
+      <c r="Z1" s="217"/>
+      <c r="AA1" s="217"/>
+      <c r="AB1" s="217"/>
+      <c r="AC1" s="217"/>
+      <c r="AD1" s="217"/>
+      <c r="AE1" s="217"/>
+      <c r="AF1" s="217"/>
+      <c r="AG1" s="217"/>
+      <c r="AH1" s="217"/>
+      <c r="AI1" s="217"/>
+      <c r="AJ1" s="217"/>
+      <c r="AK1" s="217"/>
+      <c r="AL1" s="217"/>
+      <c r="AM1" s="217"/>
+      <c r="AN1" s="217"/>
+      <c r="AO1" s="217"/>
     </row>
     <row r="2" spans="1:59" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="14" t="s">
         <v>109</v>
       </c>
       <c r="B2" s="172"/>
-      <c r="C2" s="211" t="s">
+      <c r="C2" s="225" t="s">
         <v>148</v>
       </c>
-      <c r="D2" s="211"/>
-      <c r="E2" s="211"/>
-      <c r="F2" s="211"/>
-      <c r="G2" s="211"/>
-      <c r="H2" s="211"/>
-      <c r="I2" s="211"/>
-      <c r="J2" s="211"/>
-      <c r="K2" s="211"/>
-      <c r="L2" s="211"/>
-      <c r="M2" s="211"/>
-      <c r="N2" s="211"/>
-      <c r="O2" s="211"/>
-      <c r="P2" s="211"/>
-      <c r="Q2" s="211"/>
-      <c r="R2" s="211"/>
-      <c r="S2" s="211"/>
-      <c r="T2" s="211"/>
-      <c r="U2" s="211"/>
-      <c r="V2" s="211"/>
-      <c r="W2" s="211"/>
-      <c r="X2" s="211"/>
-      <c r="Y2" s="211"/>
-      <c r="Z2" s="211"/>
-      <c r="AA2" s="211"/>
-      <c r="AB2" s="211"/>
-      <c r="AC2" s="211"/>
-      <c r="AD2" s="211"/>
-      <c r="AE2" s="211"/>
-      <c r="AF2" s="211"/>
-      <c r="AG2" s="211"/>
-      <c r="AH2" s="211"/>
-      <c r="AI2" s="211"/>
-      <c r="AJ2" s="211"/>
-      <c r="AK2" s="211"/>
-      <c r="AL2" s="211"/>
-      <c r="AM2" s="211"/>
-      <c r="AN2" s="211"/>
-      <c r="AO2" s="211"/>
+      <c r="D2" s="225"/>
+      <c r="E2" s="225"/>
+      <c r="F2" s="225"/>
+      <c r="G2" s="225"/>
+      <c r="H2" s="225"/>
+      <c r="I2" s="225"/>
+      <c r="J2" s="225"/>
+      <c r="K2" s="225"/>
+      <c r="L2" s="225"/>
+      <c r="M2" s="225"/>
+      <c r="N2" s="225"/>
+      <c r="O2" s="225"/>
+      <c r="P2" s="225"/>
+      <c r="Q2" s="225"/>
+      <c r="R2" s="225"/>
+      <c r="S2" s="225"/>
+      <c r="T2" s="225"/>
+      <c r="U2" s="225"/>
+      <c r="V2" s="225"/>
+      <c r="W2" s="225"/>
+      <c r="X2" s="225"/>
+      <c r="Y2" s="225"/>
+      <c r="Z2" s="225"/>
+      <c r="AA2" s="225"/>
+      <c r="AB2" s="225"/>
+      <c r="AC2" s="225"/>
+      <c r="AD2" s="225"/>
+      <c r="AE2" s="225"/>
+      <c r="AF2" s="225"/>
+      <c r="AG2" s="225"/>
+      <c r="AH2" s="225"/>
+      <c r="AI2" s="225"/>
+      <c r="AJ2" s="225"/>
+      <c r="AK2" s="225"/>
+      <c r="AL2" s="225"/>
+      <c r="AM2" s="225"/>
+      <c r="AN2" s="225"/>
+      <c r="AO2" s="225"/>
     </row>
     <row r="3" spans="1:59" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B3" s="208" t="s">
+      <c r="B3" s="222" t="s">
         <v>94</v>
       </c>
-      <c r="C3" s="209"/>
-      <c r="D3" s="209"/>
-      <c r="E3" s="210"/>
-      <c r="F3" s="208" t="s">
+      <c r="C3" s="223"/>
+      <c r="D3" s="223"/>
+      <c r="E3" s="224"/>
+      <c r="F3" s="222" t="s">
         <v>95</v>
       </c>
-      <c r="G3" s="209"/>
-      <c r="H3" s="209"/>
-      <c r="I3" s="210"/>
-      <c r="J3" s="208" t="s">
+      <c r="G3" s="223"/>
+      <c r="H3" s="223"/>
+      <c r="I3" s="224"/>
+      <c r="J3" s="222" t="s">
         <v>96</v>
       </c>
-      <c r="K3" s="209"/>
-      <c r="L3" s="209"/>
-      <c r="M3" s="210"/>
-      <c r="N3" s="208" t="s">
+      <c r="K3" s="223"/>
+      <c r="L3" s="223"/>
+      <c r="M3" s="224"/>
+      <c r="N3" s="222" t="s">
         <v>97</v>
       </c>
-      <c r="O3" s="209"/>
-      <c r="P3" s="209"/>
-      <c r="Q3" s="210"/>
-      <c r="R3" s="208" t="s">
+      <c r="O3" s="223"/>
+      <c r="P3" s="223"/>
+      <c r="Q3" s="224"/>
+      <c r="R3" s="222" t="s">
         <v>94</v>
       </c>
-      <c r="S3" s="209"/>
-      <c r="T3" s="209"/>
-      <c r="U3" s="210"/>
-      <c r="V3" s="208" t="s">
+      <c r="S3" s="223"/>
+      <c r="T3" s="223"/>
+      <c r="U3" s="224"/>
+      <c r="V3" s="222" t="s">
         <v>95</v>
       </c>
-      <c r="W3" s="209"/>
-      <c r="X3" s="209"/>
-      <c r="Y3" s="210"/>
-      <c r="Z3" s="208" t="s">
+      <c r="W3" s="223"/>
+      <c r="X3" s="223"/>
+      <c r="Y3" s="224"/>
+      <c r="Z3" s="222" t="s">
         <v>96</v>
       </c>
-      <c r="AA3" s="209"/>
-      <c r="AB3" s="209"/>
-      <c r="AC3" s="210"/>
-      <c r="AD3" s="208" t="s">
+      <c r="AA3" s="223"/>
+      <c r="AB3" s="223"/>
+      <c r="AC3" s="224"/>
+      <c r="AD3" s="222" t="s">
         <v>97</v>
       </c>
-      <c r="AE3" s="209"/>
-      <c r="AF3" s="209"/>
-      <c r="AG3" s="210"/>
-      <c r="AH3" s="208" t="s">
+      <c r="AE3" s="223"/>
+      <c r="AF3" s="223"/>
+      <c r="AG3" s="224"/>
+      <c r="AH3" s="222" t="s">
         <v>98</v>
       </c>
-      <c r="AI3" s="209"/>
-      <c r="AJ3" s="209"/>
-      <c r="AK3" s="210"/>
-      <c r="AL3" s="208" t="s">
+      <c r="AI3" s="223"/>
+      <c r="AJ3" s="223"/>
+      <c r="AK3" s="224"/>
+      <c r="AL3" s="222" t="s">
         <v>94</v>
       </c>
-      <c r="AM3" s="209"/>
-      <c r="AN3" s="209"/>
-      <c r="AO3" s="210"/>
-    </row>
-    <row r="4" spans="1:59" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AM3" s="223"/>
+      <c r="AN3" s="223"/>
+      <c r="AO3" s="224"/>
+    </row>
+    <row r="4" spans="1:59" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="20">
         <v>46139</v>
       </c>
-      <c r="B4" s="205" t="s">
+      <c r="B4" s="219" t="s">
         <v>99</v>
       </c>
-      <c r="C4" s="206"/>
-      <c r="D4" s="206"/>
-      <c r="E4" s="207"/>
-      <c r="F4" s="205" t="s">
+      <c r="C4" s="220"/>
+      <c r="D4" s="220"/>
+      <c r="E4" s="221"/>
+      <c r="F4" s="219" t="s">
         <v>100</v>
       </c>
-      <c r="G4" s="206"/>
-      <c r="H4" s="206"/>
-      <c r="I4" s="207"/>
-      <c r="J4" s="205" t="s">
+      <c r="G4" s="220"/>
+      <c r="H4" s="220"/>
+      <c r="I4" s="221"/>
+      <c r="J4" s="219" t="s">
         <v>101</v>
       </c>
-      <c r="K4" s="206"/>
-      <c r="L4" s="206"/>
-      <c r="M4" s="207"/>
-      <c r="N4" s="205" t="s">
+      <c r="K4" s="220"/>
+      <c r="L4" s="220"/>
+      <c r="M4" s="221"/>
+      <c r="N4" s="219" t="s">
         <v>102</v>
       </c>
-      <c r="O4" s="206"/>
-      <c r="P4" s="206"/>
-      <c r="Q4" s="207"/>
-      <c r="R4" s="205" t="s">
+      <c r="O4" s="220"/>
+      <c r="P4" s="220"/>
+      <c r="Q4" s="221"/>
+      <c r="R4" s="219" t="s">
         <v>103</v>
       </c>
-      <c r="S4" s="206"/>
-      <c r="T4" s="206"/>
-      <c r="U4" s="207"/>
-      <c r="V4" s="205" t="s">
+      <c r="S4" s="220"/>
+      <c r="T4" s="220"/>
+      <c r="U4" s="221"/>
+      <c r="V4" s="219" t="s">
         <v>104</v>
       </c>
-      <c r="W4" s="206"/>
-      <c r="X4" s="206"/>
-      <c r="Y4" s="207"/>
-      <c r="Z4" s="205" t="s">
+      <c r="W4" s="220"/>
+      <c r="X4" s="220"/>
+      <c r="Y4" s="221"/>
+      <c r="Z4" s="219" t="s">
         <v>105</v>
       </c>
-      <c r="AA4" s="206"/>
-      <c r="AB4" s="206"/>
-      <c r="AC4" s="207"/>
-      <c r="AD4" s="205" t="s">
+      <c r="AA4" s="220"/>
+      <c r="AB4" s="220"/>
+      <c r="AC4" s="221"/>
+      <c r="AD4" s="219" t="s">
         <v>106</v>
       </c>
-      <c r="AE4" s="206"/>
-      <c r="AF4" s="206"/>
-      <c r="AG4" s="207"/>
-      <c r="AH4" s="205" t="s">
+      <c r="AE4" s="220"/>
+      <c r="AF4" s="220"/>
+      <c r="AG4" s="221"/>
+      <c r="AH4" s="219" t="s">
         <v>107</v>
       </c>
-      <c r="AI4" s="206"/>
-      <c r="AJ4" s="206"/>
-      <c r="AK4" s="207"/>
-      <c r="AL4" s="205" t="s">
+      <c r="AI4" s="220"/>
+      <c r="AJ4" s="220"/>
+      <c r="AK4" s="221"/>
+      <c r="AL4" s="219" t="s">
         <v>108</v>
       </c>
-      <c r="AM4" s="206"/>
-      <c r="AN4" s="206"/>
-      <c r="AO4" s="207"/>
-    </row>
-    <row r="5" spans="1:59" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AM4" s="220"/>
+      <c r="AN4" s="220"/>
+      <c r="AO4" s="221"/>
+    </row>
+    <row r="5" spans="1:59" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="126" t="s">
         <v>114</v>
       </c>
@@ -3794,7 +3806,7 @@
       <c r="AN5" s="128"/>
       <c r="AO5" s="129"/>
     </row>
-    <row r="6" spans="1:59" s="2" customFormat="1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:59" s="2" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="125" t="s">
         <v>25</v>
       </c>
@@ -3839,7 +3851,7 @@
       <c r="AN6" s="34"/>
       <c r="AO6" s="39"/>
     </row>
-    <row r="7" spans="1:59" s="2" customFormat="1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:59" s="2" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="71" t="s">
         <v>26</v>
       </c>
@@ -3884,7 +3896,7 @@
       <c r="AN7" s="22"/>
       <c r="AO7" s="24"/>
     </row>
-    <row r="8" spans="1:59" s="2" customFormat="1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:59" s="2" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="71" t="s">
         <v>27</v>
       </c>
@@ -3929,7 +3941,7 @@
       <c r="AN8" s="22"/>
       <c r="AO8" s="24"/>
     </row>
-    <row r="9" spans="1:59" s="2" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:59" s="2" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="72" t="s">
         <v>28</v>
       </c>
@@ -3974,7 +3986,7 @@
       <c r="AN9" s="25"/>
       <c r="AO9" s="26"/>
     </row>
-    <row r="10" spans="1:59" s="2" customFormat="1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:59" s="2" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="73" t="s">
         <v>29</v>
       </c>
@@ -4019,7 +4031,7 @@
       <c r="AN10" s="98"/>
       <c r="AO10" s="113"/>
     </row>
-    <row r="11" spans="1:59" s="19" customFormat="1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:59" s="19" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="74" t="s">
         <v>30</v>
       </c>
@@ -4073,7 +4085,7 @@
       <c r="AW11" s="2"/>
       <c r="AX11" s="2"/>
     </row>
-    <row r="12" spans="1:59" s="2" customFormat="1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:59" s="2" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="75" t="s">
         <v>116</v>
       </c>
@@ -4118,7 +4130,7 @@
       <c r="AN12" s="25"/>
       <c r="AO12" s="26"/>
     </row>
-    <row r="13" spans="1:59" s="2" customFormat="1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:59" s="2" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="75" t="s">
         <v>92</v>
       </c>
@@ -4163,7 +4175,7 @@
       <c r="AN13" s="25"/>
       <c r="AO13" s="26"/>
     </row>
-    <row r="14" spans="1:59" s="19" customFormat="1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:59" s="19" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="74" t="s">
         <v>90</v>
       </c>
@@ -4226,7 +4238,7 @@
       <c r="BF14" s="2"/>
       <c r="BG14" s="2"/>
     </row>
-    <row r="15" spans="1:59" s="2" customFormat="1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:59" s="2" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="133" t="s">
         <v>118</v>
       </c>
@@ -4271,7 +4283,7 @@
       <c r="AN15" s="25"/>
       <c r="AO15" s="26"/>
     </row>
-    <row r="16" spans="1:59" s="2" customFormat="1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:59" s="2" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="133" t="s">
         <v>117</v>
       </c>
@@ -4316,7 +4328,7 @@
       <c r="AN16" s="25"/>
       <c r="AO16" s="26"/>
     </row>
-    <row r="17" spans="1:41" s="2" customFormat="1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:41" s="2" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="133" t="s">
         <v>121</v>
       </c>
@@ -4361,7 +4373,7 @@
       <c r="AN17" s="22"/>
       <c r="AO17" s="24"/>
     </row>
-    <row r="18" spans="1:41" s="2" customFormat="1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:41" s="2" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="74" t="s">
         <v>122</v>
       </c>
@@ -4406,7 +4418,7 @@
       <c r="AN18" s="25"/>
       <c r="AO18" s="26"/>
     </row>
-    <row r="19" spans="1:41" s="2" customFormat="1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:41" s="2" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="76" t="s">
         <v>31</v>
       </c>
@@ -4451,7 +4463,7 @@
       <c r="AN19" s="98"/>
       <c r="AO19" s="113"/>
     </row>
-    <row r="20" spans="1:41" s="2" customFormat="1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:41" s="2" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="77" t="s">
         <v>32</v>
       </c>
@@ -4496,7 +4508,7 @@
       <c r="AN20" s="29"/>
       <c r="AO20" s="39"/>
     </row>
-    <row r="21" spans="1:41" s="2" customFormat="1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:41" s="2" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="132" t="s">
         <v>110</v>
       </c>
@@ -4541,7 +4553,7 @@
       <c r="AN21" s="25"/>
       <c r="AO21" s="26"/>
     </row>
-    <row r="22" spans="1:41" s="2" customFormat="1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:41" s="2" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="132" t="s">
         <v>111</v>
       </c>
@@ -4586,7 +4598,7 @@
       <c r="AN22" s="25"/>
       <c r="AO22" s="26"/>
     </row>
-    <row r="23" spans="1:41" s="2" customFormat="1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:41" s="2" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="132" t="s">
         <v>112</v>
       </c>
@@ -4631,7 +4643,7 @@
       <c r="AN23" s="22"/>
       <c r="AO23" s="24"/>
     </row>
-    <row r="24" spans="1:41" s="2" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:41" s="2" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="132" t="s">
         <v>113</v>
       </c>
@@ -4876,8 +4888,8 @@
       <c r="O29" s="22"/>
       <c r="P29" s="22"/>
       <c r="Q29" s="21"/>
-      <c r="R29" s="23"/>
-      <c r="S29" s="22"/>
+      <c r="R29" s="264"/>
+      <c r="S29" s="21"/>
       <c r="T29" s="23"/>
       <c r="U29" s="24"/>
       <c r="V29" s="23"/>
@@ -5399,11 +5411,11 @@
       <c r="AH40" s="101"/>
       <c r="AI40" s="102"/>
       <c r="AJ40" s="102"/>
-      <c r="AK40" s="102"/>
-      <c r="AL40" s="101"/>
-      <c r="AM40" s="102"/>
-      <c r="AN40" s="102"/>
-      <c r="AO40" s="102"/>
+      <c r="AK40" s="197"/>
+      <c r="AL40" s="100"/>
+      <c r="AM40" s="98"/>
+      <c r="AN40" s="98"/>
+      <c r="AO40" s="113"/>
     </row>
     <row r="41" spans="1:50" s="2" customFormat="1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="86" t="s">
@@ -5673,238 +5685,238 @@
   <dimension ref="A1:BH80"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="52.7109375" customWidth="1"/>
+    <col min="1" max="1" width="48.85546875" customWidth="1"/>
     <col min="2" max="2" width="7.5703125" hidden="1" customWidth="1"/>
     <col min="3" max="42" width="2.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:51" ht="29.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="203" t="s">
+      <c r="A1" s="217" t="s">
         <v>93</v>
       </c>
-      <c r="B1" s="203"/>
-      <c r="C1" s="203"/>
-      <c r="D1" s="203"/>
-      <c r="E1" s="203"/>
-      <c r="F1" s="203"/>
-      <c r="G1" s="203"/>
-      <c r="H1" s="203"/>
-      <c r="I1" s="203"/>
-      <c r="J1" s="203"/>
-      <c r="K1" s="203"/>
-      <c r="L1" s="203"/>
-      <c r="M1" s="203"/>
-      <c r="N1" s="203"/>
-      <c r="O1" s="203"/>
-      <c r="P1" s="203"/>
-      <c r="Q1" s="203"/>
-      <c r="R1" s="203"/>
-      <c r="S1" s="203"/>
-      <c r="T1" s="203"/>
-      <c r="U1" s="203"/>
-      <c r="V1" s="203"/>
-      <c r="W1" s="203"/>
-      <c r="X1" s="203"/>
-      <c r="Y1" s="203"/>
-      <c r="Z1" s="203"/>
-      <c r="AA1" s="203"/>
-      <c r="AB1" s="203"/>
-      <c r="AC1" s="203"/>
-      <c r="AD1" s="203"/>
-      <c r="AE1" s="203"/>
-      <c r="AF1" s="203"/>
-      <c r="AG1" s="203"/>
-      <c r="AH1" s="203"/>
-      <c r="AI1" s="203"/>
-      <c r="AJ1" s="203"/>
-      <c r="AK1" s="203"/>
-      <c r="AL1" s="203"/>
-      <c r="AM1" s="203"/>
-      <c r="AN1" s="203"/>
-      <c r="AO1" s="203"/>
-      <c r="AP1" s="203"/>
+      <c r="B1" s="217"/>
+      <c r="C1" s="217"/>
+      <c r="D1" s="217"/>
+      <c r="E1" s="217"/>
+      <c r="F1" s="217"/>
+      <c r="G1" s="217"/>
+      <c r="H1" s="217"/>
+      <c r="I1" s="217"/>
+      <c r="J1" s="217"/>
+      <c r="K1" s="217"/>
+      <c r="L1" s="217"/>
+      <c r="M1" s="217"/>
+      <c r="N1" s="217"/>
+      <c r="O1" s="217"/>
+      <c r="P1" s="217"/>
+      <c r="Q1" s="217"/>
+      <c r="R1" s="217"/>
+      <c r="S1" s="217"/>
+      <c r="T1" s="217"/>
+      <c r="U1" s="217"/>
+      <c r="V1" s="217"/>
+      <c r="W1" s="217"/>
+      <c r="X1" s="217"/>
+      <c r="Y1" s="217"/>
+      <c r="Z1" s="217"/>
+      <c r="AA1" s="217"/>
+      <c r="AB1" s="217"/>
+      <c r="AC1" s="217"/>
+      <c r="AD1" s="217"/>
+      <c r="AE1" s="217"/>
+      <c r="AF1" s="217"/>
+      <c r="AG1" s="217"/>
+      <c r="AH1" s="217"/>
+      <c r="AI1" s="217"/>
+      <c r="AJ1" s="217"/>
+      <c r="AK1" s="217"/>
+      <c r="AL1" s="217"/>
+      <c r="AM1" s="217"/>
+      <c r="AN1" s="217"/>
+      <c r="AO1" s="217"/>
+      <c r="AP1" s="217"/>
     </row>
     <row r="2" spans="1:51" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="173" t="s">
         <v>109</v>
       </c>
       <c r="B2" s="14"/>
-      <c r="C2" s="204"/>
-      <c r="D2" s="204"/>
-      <c r="E2" s="204"/>
-      <c r="F2" s="204"/>
-      <c r="G2" s="204"/>
-      <c r="H2" s="204"/>
-      <c r="I2" s="204"/>
-      <c r="J2" s="204"/>
-      <c r="K2" s="204"/>
-      <c r="L2" s="204"/>
-      <c r="M2" s="204"/>
-      <c r="N2" s="204"/>
-      <c r="O2" s="204"/>
-      <c r="P2" s="204"/>
-      <c r="Q2" s="204"/>
-      <c r="R2" s="204"/>
-      <c r="S2" s="204"/>
-      <c r="T2" s="204"/>
-      <c r="U2" s="204"/>
-      <c r="V2" s="204"/>
-      <c r="W2" s="204"/>
-      <c r="X2" s="204"/>
-      <c r="Y2" s="204"/>
-      <c r="Z2" s="204"/>
-      <c r="AA2" s="204"/>
-      <c r="AB2" s="204"/>
-      <c r="AC2" s="204"/>
-      <c r="AD2" s="204"/>
-      <c r="AE2" s="204"/>
-      <c r="AF2" s="204"/>
-      <c r="AG2" s="204"/>
-      <c r="AH2" s="204"/>
-      <c r="AI2" s="204"/>
-      <c r="AJ2" s="204"/>
-      <c r="AK2" s="204"/>
-      <c r="AL2" s="204"/>
-      <c r="AM2" s="204"/>
-      <c r="AN2" s="204"/>
-      <c r="AO2" s="204"/>
-      <c r="AP2" s="204"/>
+      <c r="C2" s="218"/>
+      <c r="D2" s="218"/>
+      <c r="E2" s="218"/>
+      <c r="F2" s="218"/>
+      <c r="G2" s="218"/>
+      <c r="H2" s="218"/>
+      <c r="I2" s="218"/>
+      <c r="J2" s="218"/>
+      <c r="K2" s="218"/>
+      <c r="L2" s="218"/>
+      <c r="M2" s="218"/>
+      <c r="N2" s="218"/>
+      <c r="O2" s="218"/>
+      <c r="P2" s="218"/>
+      <c r="Q2" s="218"/>
+      <c r="R2" s="218"/>
+      <c r="S2" s="218"/>
+      <c r="T2" s="218"/>
+      <c r="U2" s="218"/>
+      <c r="V2" s="218"/>
+      <c r="W2" s="218"/>
+      <c r="X2" s="218"/>
+      <c r="Y2" s="218"/>
+      <c r="Z2" s="218"/>
+      <c r="AA2" s="218"/>
+      <c r="AB2" s="218"/>
+      <c r="AC2" s="218"/>
+      <c r="AD2" s="218"/>
+      <c r="AE2" s="218"/>
+      <c r="AF2" s="218"/>
+      <c r="AG2" s="218"/>
+      <c r="AH2" s="218"/>
+      <c r="AI2" s="218"/>
+      <c r="AJ2" s="218"/>
+      <c r="AK2" s="218"/>
+      <c r="AL2" s="218"/>
+      <c r="AM2" s="218"/>
+      <c r="AN2" s="218"/>
+      <c r="AO2" s="218"/>
+      <c r="AP2" s="218"/>
     </row>
     <row r="3" spans="1:51" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="174" t="s">
         <v>15</v>
       </c>
       <c r="B3" s="15"/>
-      <c r="C3" s="202" t="s">
+      <c r="C3" s="212" t="s">
         <v>94</v>
       </c>
-      <c r="D3" s="202"/>
-      <c r="E3" s="202"/>
-      <c r="F3" s="202"/>
-      <c r="G3" s="202" t="s">
+      <c r="D3" s="212"/>
+      <c r="E3" s="212"/>
+      <c r="F3" s="212"/>
+      <c r="G3" s="212" t="s">
         <v>95</v>
       </c>
-      <c r="H3" s="202"/>
-      <c r="I3" s="202"/>
-      <c r="J3" s="202"/>
-      <c r="K3" s="202" t="s">
+      <c r="H3" s="212"/>
+      <c r="I3" s="212"/>
+      <c r="J3" s="212"/>
+      <c r="K3" s="212" t="s">
         <v>157</v>
       </c>
-      <c r="L3" s="202"/>
-      <c r="M3" s="202"/>
-      <c r="N3" s="202"/>
-      <c r="O3" s="202" t="s">
+      <c r="L3" s="212"/>
+      <c r="M3" s="212"/>
+      <c r="N3" s="212"/>
+      <c r="O3" s="212" t="s">
         <v>97</v>
       </c>
-      <c r="P3" s="202"/>
-      <c r="Q3" s="202"/>
-      <c r="R3" s="202"/>
-      <c r="S3" s="202" t="s">
+      <c r="P3" s="212"/>
+      <c r="Q3" s="212"/>
+      <c r="R3" s="212"/>
+      <c r="S3" s="212" t="s">
         <v>94</v>
       </c>
-      <c r="T3" s="202"/>
-      <c r="U3" s="202"/>
-      <c r="V3" s="202"/>
-      <c r="W3" s="202" t="s">
+      <c r="T3" s="212"/>
+      <c r="U3" s="212"/>
+      <c r="V3" s="212"/>
+      <c r="W3" s="212" t="s">
         <v>95</v>
       </c>
-      <c r="X3" s="202"/>
-      <c r="Y3" s="202"/>
-      <c r="Z3" s="202"/>
-      <c r="AA3" s="202" t="s">
+      <c r="X3" s="212"/>
+      <c r="Y3" s="212"/>
+      <c r="Z3" s="212"/>
+      <c r="AA3" s="212" t="s">
         <v>157</v>
       </c>
-      <c r="AB3" s="202"/>
-      <c r="AC3" s="202"/>
-      <c r="AD3" s="202"/>
-      <c r="AE3" s="202" t="s">
+      <c r="AB3" s="212"/>
+      <c r="AC3" s="212"/>
+      <c r="AD3" s="212"/>
+      <c r="AE3" s="212" t="s">
         <v>97</v>
       </c>
-      <c r="AF3" s="202"/>
-      <c r="AG3" s="202"/>
-      <c r="AH3" s="202"/>
-      <c r="AI3" s="202" t="s">
+      <c r="AF3" s="212"/>
+      <c r="AG3" s="212"/>
+      <c r="AH3" s="212"/>
+      <c r="AI3" s="212" t="s">
         <v>98</v>
       </c>
-      <c r="AJ3" s="202"/>
-      <c r="AK3" s="202"/>
-      <c r="AL3" s="202"/>
-      <c r="AM3" s="202" t="s">
+      <c r="AJ3" s="212"/>
+      <c r="AK3" s="212"/>
+      <c r="AL3" s="212"/>
+      <c r="AM3" s="212" t="s">
         <v>94</v>
       </c>
-      <c r="AN3" s="202"/>
-      <c r="AO3" s="202"/>
-      <c r="AP3" s="202"/>
+      <c r="AN3" s="212"/>
+      <c r="AO3" s="212"/>
+      <c r="AP3" s="212"/>
     </row>
     <row r="4" spans="1:51" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="175" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="B4" s="20"/>
-      <c r="C4" s="196" t="s">
+      <c r="C4" s="213" t="s">
         <v>99</v>
       </c>
-      <c r="D4" s="197"/>
-      <c r="E4" s="197"/>
-      <c r="F4" s="198"/>
-      <c r="G4" s="196" t="s">
+      <c r="D4" s="214"/>
+      <c r="E4" s="214"/>
+      <c r="F4" s="215"/>
+      <c r="G4" s="213" t="s">
         <v>100</v>
       </c>
-      <c r="H4" s="197"/>
-      <c r="I4" s="197"/>
-      <c r="J4" s="198"/>
-      <c r="K4" s="196" t="s">
+      <c r="H4" s="214"/>
+      <c r="I4" s="214"/>
+      <c r="J4" s="215"/>
+      <c r="K4" s="213" t="s">
         <v>101</v>
       </c>
-      <c r="L4" s="197"/>
-      <c r="M4" s="197"/>
-      <c r="N4" s="198"/>
-      <c r="O4" s="196" t="s">
+      <c r="L4" s="214"/>
+      <c r="M4" s="214"/>
+      <c r="N4" s="215"/>
+      <c r="O4" s="213" t="s">
         <v>102</v>
       </c>
-      <c r="P4" s="197"/>
-      <c r="Q4" s="197"/>
-      <c r="R4" s="198"/>
-      <c r="S4" s="196" t="s">
+      <c r="P4" s="214"/>
+      <c r="Q4" s="214"/>
+      <c r="R4" s="215"/>
+      <c r="S4" s="213" t="s">
         <v>103</v>
       </c>
-      <c r="T4" s="197"/>
-      <c r="U4" s="197"/>
-      <c r="V4" s="198"/>
-      <c r="W4" s="196" t="s">
+      <c r="T4" s="214"/>
+      <c r="U4" s="214"/>
+      <c r="V4" s="215"/>
+      <c r="W4" s="213" t="s">
         <v>104</v>
       </c>
-      <c r="X4" s="197"/>
-      <c r="Y4" s="197"/>
-      <c r="Z4" s="198"/>
-      <c r="AA4" s="196" t="s">
+      <c r="X4" s="214"/>
+      <c r="Y4" s="214"/>
+      <c r="Z4" s="215"/>
+      <c r="AA4" s="213" t="s">
         <v>105</v>
       </c>
-      <c r="AB4" s="197"/>
-      <c r="AC4" s="197"/>
-      <c r="AD4" s="198"/>
-      <c r="AE4" s="196" t="s">
+      <c r="AB4" s="214"/>
+      <c r="AC4" s="214"/>
+      <c r="AD4" s="215"/>
+      <c r="AE4" s="213" t="s">
         <v>106</v>
       </c>
-      <c r="AF4" s="197"/>
-      <c r="AG4" s="197"/>
-      <c r="AH4" s="198"/>
-      <c r="AI4" s="196" t="s">
+      <c r="AF4" s="214"/>
+      <c r="AG4" s="214"/>
+      <c r="AH4" s="215"/>
+      <c r="AI4" s="213" t="s">
         <v>107</v>
       </c>
-      <c r="AJ4" s="197"/>
-      <c r="AK4" s="197"/>
-      <c r="AL4" s="198"/>
-      <c r="AM4" s="196" t="s">
+      <c r="AJ4" s="214"/>
+      <c r="AK4" s="214"/>
+      <c r="AL4" s="215"/>
+      <c r="AM4" s="213" t="s">
         <v>108</v>
       </c>
-      <c r="AN4" s="197"/>
-      <c r="AO4" s="197"/>
-      <c r="AP4" s="198"/>
+      <c r="AN4" s="214"/>
+      <c r="AO4" s="214"/>
+      <c r="AP4" s="215"/>
     </row>
     <row r="5" spans="1:51" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="176" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B5" s="162" t="s">
         <v>141</v>
@@ -5999,7 +6011,7 @@
       <c r="AP6" s="39"/>
     </row>
     <row r="7" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="199" t="s">
+      <c r="A7" s="210" t="s">
         <v>26</v>
       </c>
       <c r="B7" s="141" t="s">
@@ -6047,7 +6059,7 @@
       <c r="AP7" s="24"/>
     </row>
     <row r="8" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="200"/>
+      <c r="A8" s="216"/>
       <c r="B8" s="142" t="s">
         <v>133</v>
       </c>
@@ -6093,7 +6105,7 @@
       <c r="AP8" s="24"/>
     </row>
     <row r="9" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="199" t="s">
+      <c r="A9" s="210" t="s">
         <v>27</v>
       </c>
       <c r="B9" s="141" t="s">
@@ -6143,7 +6155,7 @@
       <c r="AP9" s="24"/>
     </row>
     <row r="10" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="200"/>
+      <c r="A10" s="216"/>
       <c r="B10" s="142" t="s">
         <v>133</v>
       </c>
@@ -6188,15 +6200,15 @@
       <c r="AO10" s="22"/>
       <c r="AP10" s="24"/>
     </row>
-    <row r="11" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="199" t="s">
+    <row r="11" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="210" t="s">
         <v>28</v>
       </c>
       <c r="B11" s="141" t="s">
         <v>132</v>
       </c>
       <c r="C11" s="33"/>
-      <c r="D11" s="148" t="s">
+      <c r="D11" s="183" t="s">
         <v>139</v>
       </c>
       <c r="F11" s="32"/>
@@ -6238,12 +6250,12 @@
       <c r="AP11" s="32"/>
     </row>
     <row r="12" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="201"/>
+      <c r="A12" s="211"/>
       <c r="B12" s="142" t="s">
         <v>133</v>
       </c>
       <c r="C12" s="23"/>
-      <c r="D12" s="22"/>
+      <c r="D12" s="139"/>
       <c r="E12" s="22"/>
       <c r="F12" s="24"/>
       <c r="G12" s="27"/>
@@ -6285,7 +6297,7 @@
     </row>
     <row r="13" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="178" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B13" s="164" t="s">
         <v>147</v>
@@ -6332,7 +6344,7 @@
       <c r="AP13" s="113"/>
     </row>
     <row r="14" spans="1:51" s="19" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="192" t="s">
+      <c r="A14" s="206" t="s">
         <v>30</v>
       </c>
       <c r="B14" s="141" t="s">
@@ -6389,7 +6401,7 @@
       <c r="AY14" s="2"/>
     </row>
     <row r="15" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="193"/>
+      <c r="A15" s="207"/>
       <c r="B15" s="142" t="s">
         <v>133</v>
       </c>
@@ -6435,7 +6447,7 @@
       <c r="AP15" s="30"/>
     </row>
     <row r="16" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="192" t="s">
+      <c r="A16" s="206" t="s">
         <v>116</v>
       </c>
       <c r="B16" s="141" t="s">
@@ -6483,7 +6495,7 @@
       <c r="AP16" s="137"/>
     </row>
     <row r="17" spans="1:60" s="2" customFormat="1" ht="17.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="193"/>
+      <c r="A17" s="207"/>
       <c r="B17" s="142" t="s">
         <v>133</v>
       </c>
@@ -6529,7 +6541,7 @@
       <c r="AP17" s="26"/>
     </row>
     <row r="18" spans="1:60" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="192" t="s">
+      <c r="A18" s="206" t="s">
         <v>92</v>
       </c>
       <c r="B18" s="141" t="s">
@@ -6577,7 +6589,7 @@
       <c r="AP18" s="26"/>
     </row>
     <row r="19" spans="1:60" s="2" customFormat="1" ht="17.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="193"/>
+      <c r="A19" s="207"/>
       <c r="B19" s="142" t="s">
         <v>133</v>
       </c>
@@ -6623,7 +6635,7 @@
       <c r="AP19" s="26"/>
     </row>
     <row r="20" spans="1:60" s="19" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="192" t="s">
+      <c r="A20" s="206" t="s">
         <v>90</v>
       </c>
       <c r="B20" s="141" t="s">
@@ -6689,7 +6701,7 @@
       <c r="BH20" s="2"/>
     </row>
     <row r="21" spans="1:60" s="2" customFormat="1" ht="17.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="193"/>
+      <c r="A21" s="207"/>
       <c r="B21" s="142" t="s">
         <v>133</v>
       </c>
@@ -6735,7 +6747,7 @@
       <c r="AP21" s="24"/>
     </row>
     <row r="22" spans="1:60" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="192" t="s">
+      <c r="A22" s="206" t="s">
         <v>118</v>
       </c>
       <c r="B22" s="141" t="s">
@@ -6783,7 +6795,7 @@
       <c r="AP22" s="32"/>
     </row>
     <row r="23" spans="1:60" s="2" customFormat="1" ht="17.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="193"/>
+      <c r="A23" s="207"/>
       <c r="B23" s="142" t="s">
         <v>133</v>
       </c>
@@ -6829,7 +6841,7 @@
       <c r="AP23" s="26"/>
     </row>
     <row r="24" spans="1:60" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="192" t="s">
+      <c r="A24" s="206" t="s">
         <v>152</v>
       </c>
       <c r="B24" s="141" t="s">
@@ -6879,7 +6891,7 @@
       <c r="AP24" s="26"/>
     </row>
     <row r="25" spans="1:60" s="2" customFormat="1" ht="17.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="193"/>
+      <c r="A25" s="207"/>
       <c r="B25" s="142" t="s">
         <v>133</v>
       </c>
@@ -6925,7 +6937,7 @@
       <c r="AP25" s="26"/>
     </row>
     <row r="26" spans="1:60" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="192" t="s">
+      <c r="A26" s="206" t="s">
         <v>121</v>
       </c>
       <c r="B26" s="141" t="s">
@@ -6975,7 +6987,7 @@
       <c r="AP26" s="32"/>
     </row>
     <row r="27" spans="1:60" s="2" customFormat="1" ht="17.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="193"/>
+      <c r="A27" s="207"/>
       <c r="B27" s="142" t="s">
         <v>133</v>
       </c>
@@ -7021,7 +7033,7 @@
       <c r="AP27" s="24"/>
     </row>
     <row r="28" spans="1:60" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="192" t="s">
+      <c r="A28" s="206" t="s">
         <v>122</v>
       </c>
       <c r="B28" s="141" t="s">
@@ -7069,7 +7081,7 @@
       <c r="AP28" s="32"/>
     </row>
     <row r="29" spans="1:60" s="2" customFormat="1" ht="17.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="193"/>
+      <c r="A29" s="207"/>
       <c r="B29" s="142" t="s">
         <v>133</v>
       </c>
@@ -7116,7 +7128,7 @@
     </row>
     <row r="30" spans="1:60" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="179" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="B30" s="165" t="s">
         <v>144</v>
@@ -7163,7 +7175,7 @@
       <c r="AP30" s="113"/>
     </row>
     <row r="31" spans="1:60" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="194" t="s">
+      <c r="A31" s="208" t="s">
         <v>153</v>
       </c>
       <c r="B31" s="141" t="s">
@@ -7211,7 +7223,7 @@
       <c r="AP31" s="39"/>
     </row>
     <row r="32" spans="1:60" s="2" customFormat="1" ht="17.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="191"/>
+      <c r="A32" s="202"/>
       <c r="B32" s="142" t="s">
         <v>133</v>
       </c>
@@ -7257,7 +7269,7 @@
       <c r="AP32" s="137"/>
     </row>
     <row r="33" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="190" t="s">
+      <c r="A33" s="201" t="s">
         <v>110</v>
       </c>
       <c r="B33" s="141" t="s">
@@ -7307,7 +7319,7 @@
       <c r="AP33" s="26"/>
     </row>
     <row r="34" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="191"/>
+      <c r="A34" s="202"/>
       <c r="B34" s="142" t="s">
         <v>133</v>
       </c>
@@ -7353,7 +7365,7 @@
       <c r="AP34" s="26"/>
     </row>
     <row r="35" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="190" t="s">
+      <c r="A35" s="201" t="s">
         <v>151</v>
       </c>
       <c r="B35" s="141" t="s">
@@ -7403,7 +7415,7 @@
       <c r="AP35" s="26"/>
     </row>
     <row r="36" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="195"/>
+      <c r="A36" s="209"/>
       <c r="B36" s="142" t="s">
         <v>133</v>
       </c>
@@ -7449,7 +7461,7 @@
       <c r="AP36" s="32"/>
     </row>
     <row r="37" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="190" t="s">
+      <c r="A37" s="201" t="s">
         <v>154</v>
       </c>
       <c r="B37" s="141" t="s">
@@ -7499,7 +7511,7 @@
       <c r="AP37" s="24"/>
     </row>
     <row r="38" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="191"/>
+      <c r="A38" s="202"/>
       <c r="B38" s="142" t="s">
         <v>133</v>
       </c>
@@ -7545,7 +7557,7 @@
       <c r="AP38" s="32"/>
     </row>
     <row r="39" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="190" t="s">
+      <c r="A39" s="201" t="s">
         <v>113</v>
       </c>
       <c r="B39" s="141" t="s">
@@ -7595,7 +7607,7 @@
       <c r="AP39" s="32"/>
     </row>
     <row r="40" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="191"/>
+      <c r="A40" s="202"/>
       <c r="B40" s="142" t="s">
         <v>133</v>
       </c>
@@ -7689,7 +7701,7 @@
       <c r="AP41" s="113"/>
     </row>
     <row r="42" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="187" t="s">
+      <c r="A42" s="203" t="s">
         <v>34</v>
       </c>
       <c r="B42" s="141" t="s">
@@ -7737,7 +7749,7 @@
       <c r="AP42" s="30"/>
     </row>
     <row r="43" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="188"/>
+      <c r="A43" s="204"/>
       <c r="B43" s="142" t="s">
         <v>133</v>
       </c>
@@ -7783,7 +7795,7 @@
       <c r="AP43" s="30"/>
     </row>
     <row r="44" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="187" t="s">
+      <c r="A44" s="203" t="s">
         <v>115</v>
       </c>
       <c r="B44" s="141" t="s">
@@ -7831,7 +7843,7 @@
       <c r="AP44" s="24"/>
     </row>
     <row r="45" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="188"/>
+      <c r="A45" s="204"/>
       <c r="B45" s="142" t="s">
         <v>133</v>
       </c>
@@ -7877,7 +7889,7 @@
       <c r="AP45" s="24"/>
     </row>
     <row r="46" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="187" t="s">
+      <c r="A46" s="203" t="s">
         <v>123</v>
       </c>
       <c r="B46" s="141" t="s">
@@ -7925,7 +7937,7 @@
       <c r="AP46" s="24"/>
     </row>
     <row r="47" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="188"/>
+      <c r="A47" s="204"/>
       <c r="B47" s="142" t="s">
         <v>133</v>
       </c>
@@ -7971,7 +7983,7 @@
       <c r="AP47" s="24"/>
     </row>
     <row r="48" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="187" t="s">
+      <c r="A48" s="203" t="s">
         <v>124</v>
       </c>
       <c r="B48" s="141" t="s">
@@ -8019,7 +8031,7 @@
       <c r="AP48" s="24"/>
     </row>
     <row r="49" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="188"/>
+      <c r="A49" s="204"/>
       <c r="B49" s="142" t="s">
         <v>133</v>
       </c>
@@ -8065,7 +8077,7 @@
       <c r="AP49" s="32"/>
     </row>
     <row r="50" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="187" t="s">
+      <c r="A50" s="203" t="s">
         <v>119</v>
       </c>
       <c r="B50" s="141" t="s">
@@ -8113,7 +8125,7 @@
       <c r="AP50" s="26"/>
     </row>
     <row r="51" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="188"/>
+      <c r="A51" s="204"/>
       <c r="B51" s="142" t="s">
         <v>133</v>
       </c>
@@ -8159,7 +8171,7 @@
       <c r="AP51" s="32"/>
     </row>
     <row r="52" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="187" t="s">
+      <c r="A52" s="203" t="s">
         <v>125</v>
       </c>
       <c r="B52" s="141" t="s">
@@ -8207,7 +8219,7 @@
       <c r="AP52" s="24"/>
     </row>
     <row r="53" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="188"/>
+      <c r="A53" s="204"/>
       <c r="B53" s="142" t="s">
         <v>133</v>
       </c>
@@ -8253,7 +8265,7 @@
       <c r="AP53" s="24"/>
     </row>
     <row r="54" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="187" t="s">
+      <c r="A54" s="203" t="s">
         <v>150</v>
       </c>
       <c r="B54" s="141" t="s">
@@ -8301,7 +8313,7 @@
       <c r="AP54" s="24"/>
     </row>
     <row r="55" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="188"/>
+      <c r="A55" s="204"/>
       <c r="B55" s="142" t="s">
         <v>133</v>
       </c>
@@ -8347,7 +8359,7 @@
       <c r="AP55" s="32"/>
     </row>
     <row r="56" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="187" t="s">
+      <c r="A56" s="203" t="s">
         <v>129</v>
       </c>
       <c r="B56" s="141" t="s">
@@ -8395,7 +8407,7 @@
       <c r="AP56" s="32"/>
     </row>
     <row r="57" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="188"/>
+      <c r="A57" s="204"/>
       <c r="B57" s="142" t="s">
         <v>133</v>
       </c>
@@ -8441,7 +8453,7 @@
       <c r="AP57" s="32"/>
     </row>
     <row r="58" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="187" t="s">
+      <c r="A58" s="203" t="s">
         <v>127</v>
       </c>
       <c r="B58" s="141" t="s">
@@ -8489,7 +8501,7 @@
       <c r="AP58" s="26"/>
     </row>
     <row r="59" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="188"/>
+      <c r="A59" s="204"/>
       <c r="B59" s="142" t="s">
         <v>133</v>
       </c>
@@ -8535,7 +8547,7 @@
       <c r="AP59" s="32"/>
     </row>
     <row r="60" spans="1:51" s="40" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="187" t="s">
+      <c r="A60" s="203" t="s">
         <v>128</v>
       </c>
       <c r="B60" s="141" t="s">
@@ -8592,7 +8604,7 @@
       <c r="AY60" s="2"/>
     </row>
     <row r="61" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="189"/>
+      <c r="A61" s="205"/>
       <c r="B61" s="142" t="s">
         <v>133</v>
       </c>
@@ -8639,7 +8651,7 @@
     </row>
     <row r="62" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A62" s="181" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="B62" s="167" t="s">
         <v>146</v>
@@ -8686,7 +8698,7 @@
       <c r="AP62" s="113"/>
     </row>
     <row r="63" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="184" t="s">
+      <c r="A63" s="198" t="s">
         <v>155</v>
       </c>
       <c r="B63" s="141" t="s">
@@ -8734,7 +8746,7 @@
       <c r="AP63" s="30"/>
     </row>
     <row r="64" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A64" s="185"/>
+      <c r="A64" s="199"/>
       <c r="B64" s="142" t="s">
         <v>133</v>
       </c>
@@ -8780,7 +8792,7 @@
       <c r="AP64" s="30"/>
     </row>
     <row r="65" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A65" s="184" t="s">
+      <c r="A65" s="198" t="s">
         <v>156</v>
       </c>
       <c r="B65" s="141" t="s">
@@ -8828,7 +8840,7 @@
       <c r="AP65" s="24"/>
     </row>
     <row r="66" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="185"/>
+      <c r="A66" s="199"/>
       <c r="B66" s="142" t="s">
         <v>133</v>
       </c>
@@ -8874,7 +8886,7 @@
       <c r="AP66" s="32"/>
     </row>
     <row r="67" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="184" t="s">
+      <c r="A67" s="198" t="s">
         <v>120</v>
       </c>
       <c r="B67" s="141" t="s">
@@ -8922,7 +8934,7 @@
       <c r="AP67" s="24"/>
     </row>
     <row r="68" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="186"/>
+      <c r="A68" s="200"/>
       <c r="B68" s="142" t="s">
         <v>133</v>
       </c>
@@ -8969,7 +8981,7 @@
     </row>
     <row r="69" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A69" s="182" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B69" s="168" t="s">
         <v>143</v>
@@ -9016,7 +9028,7 @@
       <c r="AP69" s="102"/>
     </row>
     <row r="70" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="260" t="s">
+      <c r="A70" s="194" t="s">
         <v>130</v>
       </c>
       <c r="B70" s="141" t="s">
@@ -9064,7 +9076,7 @@
       <c r="AP70" s="91"/>
     </row>
     <row r="71" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="261"/>
+      <c r="A71" s="195"/>
       <c r="B71" s="142" t="s">
         <v>133</v>
       </c>
@@ -9110,7 +9122,7 @@
       <c r="AP71" s="91"/>
     </row>
     <row r="72" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="260" t="s">
+      <c r="A72" s="194" t="s">
         <v>131</v>
       </c>
       <c r="B72" s="141" t="s">
@@ -9158,7 +9170,7 @@
       <c r="AP72" s="18"/>
     </row>
     <row r="73" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A73" s="261"/>
+      <c r="A73" s="195"/>
       <c r="B73" s="142" t="s">
         <v>133</v>
       </c>
@@ -9204,7 +9216,7 @@
       <c r="AP73" s="18"/>
     </row>
     <row r="74" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A74" s="260" t="s">
+      <c r="A74" s="194" t="s">
         <v>135</v>
       </c>
       <c r="B74" s="141" t="s">
@@ -9254,7 +9266,7 @@
       <c r="AP74" s="18"/>
     </row>
     <row r="75" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A75" s="261"/>
+      <c r="A75" s="195"/>
       <c r="B75" s="142" t="s">
         <v>133</v>
       </c>
@@ -9300,7 +9312,7 @@
       <c r="AP75" s="18"/>
     </row>
     <row r="76" spans="1:42" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A76" s="260" t="s">
+      <c r="A76" s="194" t="s">
         <v>136</v>
       </c>
       <c r="B76" s="141" t="s">
@@ -9343,7 +9355,7 @@
       <c r="AK76" s="155" t="s">
         <v>139</v>
       </c>
-      <c r="AL76" s="256" t="s">
+      <c r="AL76" s="190" t="s">
         <v>139</v>
       </c>
       <c r="AM76" s="23"/>
@@ -9352,7 +9364,7 @@
       <c r="AP76" s="18"/>
     </row>
     <row r="77" spans="1:42" ht="17.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A77" s="261"/>
+      <c r="A77" s="195"/>
       <c r="B77" s="142" t="s">
         <v>133</v>
       </c>
@@ -9398,7 +9410,7 @@
       <c r="AP77" s="145"/>
     </row>
     <row r="78" spans="1:42" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="260" t="s">
+      <c r="A78" s="194" t="s">
         <v>137</v>
       </c>
       <c r="B78" s="141" t="s">
@@ -9439,7 +9451,7 @@
       <c r="AI78" s="27"/>
       <c r="AJ78" s="43"/>
       <c r="AK78" s="25"/>
-      <c r="AL78" s="257" t="s">
+      <c r="AL78" s="191" t="s">
         <v>139</v>
       </c>
       <c r="AM78" s="27"/>
@@ -9448,54 +9460,54 @@
       <c r="AP78" s="44"/>
     </row>
     <row r="79" spans="1:42" ht="17.100000000000001" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A79" s="261"/>
+      <c r="A79" s="195"/>
       <c r="B79" s="142" t="s">
         <v>133</v>
       </c>
       <c r="C79" s="109"/>
-      <c r="D79" s="254"/>
+      <c r="D79" s="188"/>
       <c r="E79" s="90"/>
-      <c r="F79" s="255"/>
+      <c r="F79" s="189"/>
       <c r="G79" s="109"/>
-      <c r="H79" s="254"/>
+      <c r="H79" s="188"/>
       <c r="I79" s="90"/>
-      <c r="J79" s="255"/>
+      <c r="J79" s="189"/>
       <c r="K79" s="109"/>
-      <c r="L79" s="254"/>
+      <c r="L79" s="188"/>
       <c r="M79" s="90"/>
-      <c r="N79" s="255"/>
+      <c r="N79" s="189"/>
       <c r="O79" s="109"/>
-      <c r="P79" s="254"/>
+      <c r="P79" s="188"/>
       <c r="Q79" s="90"/>
-      <c r="R79" s="255"/>
+      <c r="R79" s="189"/>
       <c r="S79" s="109"/>
-      <c r="T79" s="254"/>
+      <c r="T79" s="188"/>
       <c r="U79" s="90"/>
-      <c r="V79" s="255"/>
+      <c r="V79" s="189"/>
       <c r="W79" s="90"/>
-      <c r="X79" s="254"/>
+      <c r="X79" s="188"/>
       <c r="Y79" s="90"/>
-      <c r="Z79" s="255"/>
+      <c r="Z79" s="189"/>
       <c r="AA79" s="90"/>
-      <c r="AB79" s="254"/>
+      <c r="AB79" s="188"/>
       <c r="AC79" s="90"/>
-      <c r="AD79" s="255"/>
+      <c r="AD79" s="189"/>
       <c r="AE79" s="109"/>
-      <c r="AF79" s="254"/>
+      <c r="AF79" s="188"/>
       <c r="AG79" s="90"/>
-      <c r="AH79" s="255"/>
+      <c r="AH79" s="189"/>
       <c r="AI79" s="109"/>
-      <c r="AJ79" s="254"/>
+      <c r="AJ79" s="188"/>
       <c r="AK79" s="90"/>
-      <c r="AL79" s="255"/>
+      <c r="AL79" s="189"/>
       <c r="AM79" s="109"/>
-      <c r="AN79" s="254"/>
+      <c r="AN79" s="188"/>
       <c r="AO79" s="90"/>
-      <c r="AP79" s="255"/>
+      <c r="AP79" s="189"/>
     </row>
     <row r="80" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A80" s="250" t="s">
-        <v>166</v>
+      <c r="A80" s="184" t="s">
+        <v>167</v>
       </c>
       <c r="B80" s="168" t="s">
         <v>143</v>
@@ -9536,10 +9548,10 @@
       <c r="AJ80" s="97"/>
       <c r="AK80" s="98"/>
       <c r="AL80" s="99"/>
-      <c r="AM80" s="251"/>
-      <c r="AN80" s="252"/>
-      <c r="AO80" s="251"/>
-      <c r="AP80" s="253"/>
+      <c r="AM80" s="185"/>
+      <c r="AN80" s="186"/>
+      <c r="AO80" s="185"/>
+      <c r="AP80" s="187"/>
     </row>
   </sheetData>
   <mergeCells count="52">
@@ -9581,6 +9593,8 @@
     <mergeCell ref="A31:A32"/>
     <mergeCell ref="A33:A34"/>
     <mergeCell ref="A35:A36"/>
+    <mergeCell ref="A65:A66"/>
+    <mergeCell ref="A67:A68"/>
     <mergeCell ref="A63:A64"/>
     <mergeCell ref="A39:A40"/>
     <mergeCell ref="A42:A43"/>
@@ -9593,8 +9607,6 @@
     <mergeCell ref="A56:A57"/>
     <mergeCell ref="A58:A59"/>
     <mergeCell ref="A60:A61"/>
-    <mergeCell ref="A65:A66"/>
-    <mergeCell ref="A67:A68"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.35" right="0.35" top="0.35" bottom="0.5" header="0.3" footer="0.3"/>
@@ -9619,232 +9631,232 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:51" ht="29.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="203" t="s">
+      <c r="A1" s="217" t="s">
         <v>93</v>
       </c>
-      <c r="B1" s="203"/>
-      <c r="C1" s="203"/>
-      <c r="D1" s="203"/>
-      <c r="E1" s="203"/>
-      <c r="F1" s="203"/>
-      <c r="G1" s="203"/>
-      <c r="H1" s="203"/>
-      <c r="I1" s="203"/>
-      <c r="J1" s="203"/>
-      <c r="K1" s="203"/>
-      <c r="L1" s="203"/>
-      <c r="M1" s="203"/>
-      <c r="N1" s="203"/>
-      <c r="O1" s="203"/>
-      <c r="P1" s="203"/>
-      <c r="Q1" s="203"/>
-      <c r="R1" s="203"/>
-      <c r="S1" s="203"/>
-      <c r="T1" s="203"/>
-      <c r="U1" s="203"/>
-      <c r="V1" s="203"/>
-      <c r="W1" s="203"/>
-      <c r="X1" s="203"/>
-      <c r="Y1" s="203"/>
-      <c r="Z1" s="203"/>
-      <c r="AA1" s="203"/>
-      <c r="AB1" s="203"/>
-      <c r="AC1" s="203"/>
-      <c r="AD1" s="203"/>
-      <c r="AE1" s="203"/>
-      <c r="AF1" s="203"/>
-      <c r="AG1" s="203"/>
-      <c r="AH1" s="203"/>
-      <c r="AI1" s="203"/>
-      <c r="AJ1" s="203"/>
-      <c r="AK1" s="203"/>
-      <c r="AL1" s="203"/>
-      <c r="AM1" s="203"/>
-      <c r="AN1" s="203"/>
-      <c r="AO1" s="203"/>
-      <c r="AP1" s="203"/>
+      <c r="B1" s="217"/>
+      <c r="C1" s="217"/>
+      <c r="D1" s="217"/>
+      <c r="E1" s="217"/>
+      <c r="F1" s="217"/>
+      <c r="G1" s="217"/>
+      <c r="H1" s="217"/>
+      <c r="I1" s="217"/>
+      <c r="J1" s="217"/>
+      <c r="K1" s="217"/>
+      <c r="L1" s="217"/>
+      <c r="M1" s="217"/>
+      <c r="N1" s="217"/>
+      <c r="O1" s="217"/>
+      <c r="P1" s="217"/>
+      <c r="Q1" s="217"/>
+      <c r="R1" s="217"/>
+      <c r="S1" s="217"/>
+      <c r="T1" s="217"/>
+      <c r="U1" s="217"/>
+      <c r="V1" s="217"/>
+      <c r="W1" s="217"/>
+      <c r="X1" s="217"/>
+      <c r="Y1" s="217"/>
+      <c r="Z1" s="217"/>
+      <c r="AA1" s="217"/>
+      <c r="AB1" s="217"/>
+      <c r="AC1" s="217"/>
+      <c r="AD1" s="217"/>
+      <c r="AE1" s="217"/>
+      <c r="AF1" s="217"/>
+      <c r="AG1" s="217"/>
+      <c r="AH1" s="217"/>
+      <c r="AI1" s="217"/>
+      <c r="AJ1" s="217"/>
+      <c r="AK1" s="217"/>
+      <c r="AL1" s="217"/>
+      <c r="AM1" s="217"/>
+      <c r="AN1" s="217"/>
+      <c r="AO1" s="217"/>
+      <c r="AP1" s="217"/>
     </row>
     <row r="2" spans="1:51" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="14" t="s">
         <v>109</v>
       </c>
       <c r="B2" s="14"/>
-      <c r="C2" s="227" t="s">
+      <c r="C2" s="241" t="s">
         <v>140</v>
       </c>
-      <c r="D2" s="228"/>
-      <c r="E2" s="227" t="s">
+      <c r="D2" s="242"/>
+      <c r="E2" s="241" t="s">
         <v>149</v>
       </c>
-      <c r="F2" s="229"/>
-      <c r="G2" s="229"/>
-      <c r="H2" s="229"/>
-      <c r="I2" s="229"/>
-      <c r="J2" s="229"/>
-      <c r="K2" s="229"/>
-      <c r="L2" s="229"/>
-      <c r="M2" s="229"/>
-      <c r="N2" s="229"/>
-      <c r="O2" s="229"/>
-      <c r="P2" s="229"/>
-      <c r="Q2" s="229"/>
-      <c r="R2" s="229"/>
-      <c r="S2" s="229"/>
-      <c r="T2" s="229"/>
-      <c r="U2" s="229"/>
-      <c r="V2" s="229"/>
-      <c r="W2" s="229"/>
-      <c r="X2" s="229"/>
-      <c r="Y2" s="229"/>
-      <c r="Z2" s="229"/>
-      <c r="AA2" s="229"/>
-      <c r="AB2" s="229"/>
-      <c r="AC2" s="229"/>
-      <c r="AD2" s="229"/>
-      <c r="AE2" s="229"/>
-      <c r="AF2" s="229"/>
-      <c r="AG2" s="229"/>
-      <c r="AH2" s="229"/>
-      <c r="AI2" s="229"/>
-      <c r="AJ2" s="229"/>
-      <c r="AK2" s="229"/>
-      <c r="AL2" s="229"/>
-      <c r="AM2" s="229"/>
-      <c r="AN2" s="229"/>
-      <c r="AO2" s="229"/>
-      <c r="AP2" s="228"/>
+      <c r="F2" s="243"/>
+      <c r="G2" s="243"/>
+      <c r="H2" s="243"/>
+      <c r="I2" s="243"/>
+      <c r="J2" s="243"/>
+      <c r="K2" s="243"/>
+      <c r="L2" s="243"/>
+      <c r="M2" s="243"/>
+      <c r="N2" s="243"/>
+      <c r="O2" s="243"/>
+      <c r="P2" s="243"/>
+      <c r="Q2" s="243"/>
+      <c r="R2" s="243"/>
+      <c r="S2" s="243"/>
+      <c r="T2" s="243"/>
+      <c r="U2" s="243"/>
+      <c r="V2" s="243"/>
+      <c r="W2" s="243"/>
+      <c r="X2" s="243"/>
+      <c r="Y2" s="243"/>
+      <c r="Z2" s="243"/>
+      <c r="AA2" s="243"/>
+      <c r="AB2" s="243"/>
+      <c r="AC2" s="243"/>
+      <c r="AD2" s="243"/>
+      <c r="AE2" s="243"/>
+      <c r="AF2" s="243"/>
+      <c r="AG2" s="243"/>
+      <c r="AH2" s="243"/>
+      <c r="AI2" s="243"/>
+      <c r="AJ2" s="243"/>
+      <c r="AK2" s="243"/>
+      <c r="AL2" s="243"/>
+      <c r="AM2" s="243"/>
+      <c r="AN2" s="243"/>
+      <c r="AO2" s="243"/>
+      <c r="AP2" s="242"/>
     </row>
     <row r="3" spans="1:51" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
         <v>15</v>
       </c>
       <c r="B3" s="15"/>
-      <c r="C3" s="208" t="s">
+      <c r="C3" s="222" t="s">
         <v>94</v>
       </c>
-      <c r="D3" s="209"/>
-      <c r="E3" s="209"/>
-      <c r="F3" s="210"/>
-      <c r="G3" s="208" t="s">
+      <c r="D3" s="223"/>
+      <c r="E3" s="223"/>
+      <c r="F3" s="224"/>
+      <c r="G3" s="222" t="s">
         <v>95</v>
       </c>
-      <c r="H3" s="209"/>
-      <c r="I3" s="209"/>
-      <c r="J3" s="210"/>
-      <c r="K3" s="208" t="s">
+      <c r="H3" s="223"/>
+      <c r="I3" s="223"/>
+      <c r="J3" s="224"/>
+      <c r="K3" s="222" t="s">
         <v>96</v>
       </c>
-      <c r="L3" s="209"/>
-      <c r="M3" s="209"/>
-      <c r="N3" s="210"/>
-      <c r="O3" s="208" t="s">
+      <c r="L3" s="223"/>
+      <c r="M3" s="223"/>
+      <c r="N3" s="224"/>
+      <c r="O3" s="222" t="s">
         <v>97</v>
       </c>
-      <c r="P3" s="209"/>
-      <c r="Q3" s="209"/>
-      <c r="R3" s="210"/>
-      <c r="S3" s="208" t="s">
+      <c r="P3" s="223"/>
+      <c r="Q3" s="223"/>
+      <c r="R3" s="224"/>
+      <c r="S3" s="222" t="s">
         <v>94</v>
       </c>
-      <c r="T3" s="209"/>
-      <c r="U3" s="209"/>
-      <c r="V3" s="210"/>
-      <c r="W3" s="208" t="s">
+      <c r="T3" s="223"/>
+      <c r="U3" s="223"/>
+      <c r="V3" s="224"/>
+      <c r="W3" s="222" t="s">
         <v>95</v>
       </c>
-      <c r="X3" s="209"/>
-      <c r="Y3" s="209"/>
-      <c r="Z3" s="210"/>
-      <c r="AA3" s="208" t="s">
+      <c r="X3" s="223"/>
+      <c r="Y3" s="223"/>
+      <c r="Z3" s="224"/>
+      <c r="AA3" s="222" t="s">
         <v>96</v>
       </c>
-      <c r="AB3" s="209"/>
-      <c r="AC3" s="209"/>
-      <c r="AD3" s="210"/>
-      <c r="AE3" s="208" t="s">
+      <c r="AB3" s="223"/>
+      <c r="AC3" s="223"/>
+      <c r="AD3" s="224"/>
+      <c r="AE3" s="222" t="s">
         <v>97</v>
       </c>
-      <c r="AF3" s="209"/>
-      <c r="AG3" s="209"/>
-      <c r="AH3" s="210"/>
-      <c r="AI3" s="208" t="s">
+      <c r="AF3" s="223"/>
+      <c r="AG3" s="223"/>
+      <c r="AH3" s="224"/>
+      <c r="AI3" s="222" t="s">
         <v>98</v>
       </c>
-      <c r="AJ3" s="209"/>
-      <c r="AK3" s="209"/>
-      <c r="AL3" s="210"/>
-      <c r="AM3" s="208" t="s">
+      <c r="AJ3" s="223"/>
+      <c r="AK3" s="223"/>
+      <c r="AL3" s="224"/>
+      <c r="AM3" s="222" t="s">
         <v>94</v>
       </c>
-      <c r="AN3" s="209"/>
-      <c r="AO3" s="209"/>
-      <c r="AP3" s="210"/>
+      <c r="AN3" s="223"/>
+      <c r="AO3" s="223"/>
+      <c r="AP3" s="224"/>
     </row>
     <row r="4" spans="1:51" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="20">
         <v>46139</v>
       </c>
       <c r="B4" s="20"/>
-      <c r="C4" s="205" t="s">
+      <c r="C4" s="219" t="s">
         <v>99</v>
       </c>
-      <c r="D4" s="206"/>
-      <c r="E4" s="206"/>
-      <c r="F4" s="207"/>
-      <c r="G4" s="205" t="s">
+      <c r="D4" s="220"/>
+      <c r="E4" s="220"/>
+      <c r="F4" s="221"/>
+      <c r="G4" s="219" t="s">
         <v>100</v>
       </c>
-      <c r="H4" s="206"/>
-      <c r="I4" s="206"/>
-      <c r="J4" s="207"/>
-      <c r="K4" s="205" t="s">
+      <c r="H4" s="220"/>
+      <c r="I4" s="220"/>
+      <c r="J4" s="221"/>
+      <c r="K4" s="219" t="s">
         <v>101</v>
       </c>
-      <c r="L4" s="206"/>
-      <c r="M4" s="206"/>
-      <c r="N4" s="207"/>
-      <c r="O4" s="205" t="s">
+      <c r="L4" s="220"/>
+      <c r="M4" s="220"/>
+      <c r="N4" s="221"/>
+      <c r="O4" s="219" t="s">
         <v>102</v>
       </c>
-      <c r="P4" s="206"/>
-      <c r="Q4" s="206"/>
-      <c r="R4" s="207"/>
-      <c r="S4" s="205" t="s">
+      <c r="P4" s="220"/>
+      <c r="Q4" s="220"/>
+      <c r="R4" s="221"/>
+      <c r="S4" s="219" t="s">
         <v>103</v>
       </c>
-      <c r="T4" s="206"/>
-      <c r="U4" s="206"/>
-      <c r="V4" s="207"/>
-      <c r="W4" s="205" t="s">
+      <c r="T4" s="220"/>
+      <c r="U4" s="220"/>
+      <c r="V4" s="221"/>
+      <c r="W4" s="219" t="s">
         <v>104</v>
       </c>
-      <c r="X4" s="206"/>
-      <c r="Y4" s="206"/>
-      <c r="Z4" s="207"/>
-      <c r="AA4" s="205" t="s">
+      <c r="X4" s="220"/>
+      <c r="Y4" s="220"/>
+      <c r="Z4" s="221"/>
+      <c r="AA4" s="219" t="s">
         <v>105</v>
       </c>
-      <c r="AB4" s="206"/>
-      <c r="AC4" s="206"/>
-      <c r="AD4" s="207"/>
-      <c r="AE4" s="205" t="s">
+      <c r="AB4" s="220"/>
+      <c r="AC4" s="220"/>
+      <c r="AD4" s="221"/>
+      <c r="AE4" s="219" t="s">
         <v>106</v>
       </c>
-      <c r="AF4" s="206"/>
-      <c r="AG4" s="206"/>
-      <c r="AH4" s="207"/>
-      <c r="AI4" s="205" t="s">
+      <c r="AF4" s="220"/>
+      <c r="AG4" s="220"/>
+      <c r="AH4" s="221"/>
+      <c r="AI4" s="219" t="s">
         <v>107</v>
       </c>
-      <c r="AJ4" s="206"/>
-      <c r="AK4" s="206"/>
-      <c r="AL4" s="207"/>
-      <c r="AM4" s="205" t="s">
+      <c r="AJ4" s="220"/>
+      <c r="AK4" s="220"/>
+      <c r="AL4" s="221"/>
+      <c r="AM4" s="219" t="s">
         <v>108</v>
       </c>
-      <c r="AN4" s="206"/>
-      <c r="AO4" s="206"/>
-      <c r="AP4" s="207"/>
+      <c r="AN4" s="220"/>
+      <c r="AO4" s="220"/>
+      <c r="AP4" s="221"/>
     </row>
     <row r="5" spans="1:51" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="126" t="s">
@@ -9943,7 +9955,7 @@
       <c r="AP6" s="39"/>
     </row>
     <row r="7" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="214" t="s">
+      <c r="A7" s="230" t="s">
         <v>26</v>
       </c>
       <c r="B7" s="141" t="s">
@@ -9991,7 +10003,7 @@
       <c r="AP7" s="24"/>
     </row>
     <row r="8" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="215"/>
+      <c r="A8" s="231"/>
       <c r="B8" s="142" t="s">
         <v>133</v>
       </c>
@@ -10037,7 +10049,7 @@
       <c r="AP8" s="24"/>
     </row>
     <row r="9" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="214" t="s">
+      <c r="A9" s="230" t="s">
         <v>27</v>
       </c>
       <c r="B9" s="141" t="s">
@@ -10087,7 +10099,7 @@
       <c r="AP9" s="24"/>
     </row>
     <row r="10" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="215"/>
+      <c r="A10" s="231"/>
       <c r="B10" s="142" t="s">
         <v>133</v>
       </c>
@@ -10135,7 +10147,7 @@
       <c r="AP10" s="24"/>
     </row>
     <row r="11" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="214" t="s">
+      <c r="A11" s="230" t="s">
         <v>28</v>
       </c>
       <c r="B11" s="141" t="s">
@@ -10184,7 +10196,7 @@
       <c r="AP11" s="32"/>
     </row>
     <row r="12" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="222"/>
+      <c r="A12" s="236"/>
       <c r="B12" s="142" t="s">
         <v>133</v>
       </c>
@@ -10280,7 +10292,7 @@
       <c r="AP13" s="113"/>
     </row>
     <row r="14" spans="1:51" s="19" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="220" t="s">
+      <c r="A14" s="226" t="s">
         <v>30</v>
       </c>
       <c r="B14" s="141" t="s">
@@ -10337,7 +10349,7 @@
       <c r="AY14" s="2"/>
     </row>
     <row r="15" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="221"/>
+      <c r="A15" s="227"/>
       <c r="B15" s="142" t="s">
         <v>133</v>
       </c>
@@ -10385,7 +10397,7 @@
       <c r="AP15" s="30"/>
     </row>
     <row r="16" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="220" t="s">
+      <c r="A16" s="226" t="s">
         <v>116</v>
       </c>
       <c r="B16" s="141" t="s">
@@ -10433,7 +10445,7 @@
       <c r="AP16" s="137"/>
     </row>
     <row r="17" spans="1:60" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="221"/>
+      <c r="A17" s="227"/>
       <c r="B17" s="142" t="s">
         <v>133</v>
       </c>
@@ -10481,7 +10493,7 @@
       <c r="AP17" s="26"/>
     </row>
     <row r="18" spans="1:60" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="220" t="s">
+      <c r="A18" s="226" t="s">
         <v>92</v>
       </c>
       <c r="B18" s="141" t="s">
@@ -10529,7 +10541,7 @@
       <c r="AP18" s="26"/>
     </row>
     <row r="19" spans="1:60" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="221"/>
+      <c r="A19" s="227"/>
       <c r="B19" s="142" t="s">
         <v>133</v>
       </c>
@@ -10577,7 +10589,7 @@
       <c r="AP19" s="26"/>
     </row>
     <row r="20" spans="1:60" s="19" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="220" t="s">
+      <c r="A20" s="226" t="s">
         <v>90</v>
       </c>
       <c r="B20" s="141" t="s">
@@ -10643,7 +10655,7 @@
       <c r="BH20" s="2"/>
     </row>
     <row r="21" spans="1:60" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="221"/>
+      <c r="A21" s="227"/>
       <c r="B21" s="142" t="s">
         <v>133</v>
       </c>
@@ -10691,7 +10703,7 @@
       <c r="AP21" s="24"/>
     </row>
     <row r="22" spans="1:60" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="220" t="s">
+      <c r="A22" s="226" t="s">
         <v>118</v>
       </c>
       <c r="B22" s="141" t="s">
@@ -10739,7 +10751,7 @@
       <c r="AP22" s="32"/>
     </row>
     <row r="23" spans="1:60" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="221"/>
+      <c r="A23" s="227"/>
       <c r="B23" s="142" t="s">
         <v>133</v>
       </c>
@@ -10785,7 +10797,7 @@
       <c r="AP23" s="26"/>
     </row>
     <row r="24" spans="1:60" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="220" t="s">
+      <c r="A24" s="226" t="s">
         <v>117</v>
       </c>
       <c r="B24" s="141" t="s">
@@ -10835,7 +10847,7 @@
       <c r="AP24" s="26"/>
     </row>
     <row r="25" spans="1:60" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="221"/>
+      <c r="A25" s="227"/>
       <c r="B25" s="142" t="s">
         <v>133</v>
       </c>
@@ -10881,7 +10893,7 @@
       <c r="AP25" s="26"/>
     </row>
     <row r="26" spans="1:60" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="220" t="s">
+      <c r="A26" s="226" t="s">
         <v>121</v>
       </c>
       <c r="B26" s="141" t="s">
@@ -10931,7 +10943,7 @@
       <c r="AP26" s="32"/>
     </row>
     <row r="27" spans="1:60" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="221"/>
+      <c r="A27" s="227"/>
       <c r="B27" s="142" t="s">
         <v>133</v>
       </c>
@@ -10977,7 +10989,7 @@
       <c r="AP27" s="24"/>
     </row>
     <row r="28" spans="1:60" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="220" t="s">
+      <c r="A28" s="226" t="s">
         <v>122</v>
       </c>
       <c r="B28" s="141" t="s">
@@ -11025,7 +11037,7 @@
       <c r="AP28" s="32"/>
     </row>
     <row r="29" spans="1:60" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="221"/>
+      <c r="A29" s="227"/>
       <c r="B29" s="142" t="s">
         <v>133</v>
       </c>
@@ -11119,7 +11131,7 @@
       <c r="AP30" s="113"/>
     </row>
     <row r="31" spans="1:60" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="219" t="s">
+      <c r="A31" s="235" t="s">
         <v>32</v>
       </c>
       <c r="B31" s="141" t="s">
@@ -11167,7 +11179,7 @@
       <c r="AP31" s="39"/>
     </row>
     <row r="32" spans="1:60" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="217"/>
+      <c r="A32" s="233"/>
       <c r="B32" s="142" t="s">
         <v>133</v>
       </c>
@@ -11213,7 +11225,7 @@
       <c r="AP32" s="137"/>
     </row>
     <row r="33" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="216" t="s">
+      <c r="A33" s="232" t="s">
         <v>110</v>
       </c>
       <c r="B33" s="141" t="s">
@@ -11263,7 +11275,7 @@
       <c r="AP33" s="26"/>
     </row>
     <row r="34" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="217"/>
+      <c r="A34" s="233"/>
       <c r="B34" s="142" t="s">
         <v>133</v>
       </c>
@@ -11309,7 +11321,7 @@
       <c r="AP34" s="26"/>
     </row>
     <row r="35" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="216" t="s">
+      <c r="A35" s="232" t="s">
         <v>111</v>
       </c>
       <c r="B35" s="141" t="s">
@@ -11359,7 +11371,7 @@
       <c r="AP35" s="26"/>
     </row>
     <row r="36" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="218"/>
+      <c r="A36" s="234"/>
       <c r="B36" s="142" t="s">
         <v>133</v>
       </c>
@@ -11405,7 +11417,7 @@
       <c r="AP36" s="32"/>
     </row>
     <row r="37" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="216" t="s">
+      <c r="A37" s="232" t="s">
         <v>112</v>
       </c>
       <c r="B37" s="141" t="s">
@@ -11455,7 +11467,7 @@
       <c r="AP37" s="24"/>
     </row>
     <row r="38" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="217"/>
+      <c r="A38" s="233"/>
       <c r="B38" s="142" t="s">
         <v>133</v>
       </c>
@@ -11501,7 +11513,7 @@
       <c r="AP38" s="32"/>
     </row>
     <row r="39" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="216" t="s">
+      <c r="A39" s="232" t="s">
         <v>113</v>
       </c>
       <c r="B39" s="141" t="s">
@@ -11551,7 +11563,7 @@
       <c r="AP39" s="32"/>
     </row>
     <row r="40" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="217"/>
+      <c r="A40" s="233"/>
       <c r="B40" s="142" t="s">
         <v>133</v>
       </c>
@@ -11645,7 +11657,7 @@
       <c r="AP41" s="113"/>
     </row>
     <row r="42" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="212" t="s">
+      <c r="A42" s="228" t="s">
         <v>34</v>
       </c>
       <c r="B42" s="141" t="s">
@@ -11693,7 +11705,7 @@
       <c r="AP42" s="30"/>
     </row>
     <row r="43" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="213"/>
+      <c r="A43" s="229"/>
       <c r="B43" s="142" t="s">
         <v>133</v>
       </c>
@@ -11739,7 +11751,7 @@
       <c r="AP43" s="30"/>
     </row>
     <row r="44" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="212" t="s">
+      <c r="A44" s="228" t="s">
         <v>115</v>
       </c>
       <c r="B44" s="141" t="s">
@@ -11787,7 +11799,7 @@
       <c r="AP44" s="24"/>
     </row>
     <row r="45" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="213"/>
+      <c r="A45" s="229"/>
       <c r="B45" s="142" t="s">
         <v>133</v>
       </c>
@@ -11833,7 +11845,7 @@
       <c r="AP45" s="24"/>
     </row>
     <row r="46" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="212" t="s">
+      <c r="A46" s="228" t="s">
         <v>123</v>
       </c>
       <c r="B46" s="141" t="s">
@@ -11881,7 +11893,7 @@
       <c r="AP46" s="24"/>
     </row>
     <row r="47" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="213"/>
+      <c r="A47" s="229"/>
       <c r="B47" s="142" t="s">
         <v>133</v>
       </c>
@@ -11927,7 +11939,7 @@
       <c r="AP47" s="24"/>
     </row>
     <row r="48" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="212" t="s">
+      <c r="A48" s="228" t="s">
         <v>124</v>
       </c>
       <c r="B48" s="141" t="s">
@@ -11975,7 +11987,7 @@
       <c r="AP48" s="24"/>
     </row>
     <row r="49" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="213"/>
+      <c r="A49" s="229"/>
       <c r="B49" s="142" t="s">
         <v>133</v>
       </c>
@@ -12021,7 +12033,7 @@
       <c r="AP49" s="32"/>
     </row>
     <row r="50" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="212" t="s">
+      <c r="A50" s="228" t="s">
         <v>119</v>
       </c>
       <c r="B50" s="141" t="s">
@@ -12069,7 +12081,7 @@
       <c r="AP50" s="26"/>
     </row>
     <row r="51" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="213"/>
+      <c r="A51" s="229"/>
       <c r="B51" s="142" t="s">
         <v>133</v>
       </c>
@@ -12115,7 +12127,7 @@
       <c r="AP51" s="32"/>
     </row>
     <row r="52" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="212" t="s">
+      <c r="A52" s="228" t="s">
         <v>125</v>
       </c>
       <c r="B52" s="141" t="s">
@@ -12163,7 +12175,7 @@
       <c r="AP52" s="24"/>
     </row>
     <row r="53" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="213"/>
+      <c r="A53" s="229"/>
       <c r="B53" s="142" t="s">
         <v>133</v>
       </c>
@@ -12209,7 +12221,7 @@
       <c r="AP53" s="24"/>
     </row>
     <row r="54" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="212" t="s">
+      <c r="A54" s="228" t="s">
         <v>126</v>
       </c>
       <c r="B54" s="141" t="s">
@@ -12257,7 +12269,7 @@
       <c r="AP54" s="24"/>
     </row>
     <row r="55" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="213"/>
+      <c r="A55" s="229"/>
       <c r="B55" s="142" t="s">
         <v>133</v>
       </c>
@@ -12303,7 +12315,7 @@
       <c r="AP55" s="32"/>
     </row>
     <row r="56" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="212" t="s">
+      <c r="A56" s="228" t="s">
         <v>129</v>
       </c>
       <c r="B56" s="141" t="s">
@@ -12351,7 +12363,7 @@
       <c r="AP56" s="32"/>
     </row>
     <row r="57" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="213"/>
+      <c r="A57" s="229"/>
       <c r="B57" s="142" t="s">
         <v>133</v>
       </c>
@@ -12397,7 +12409,7 @@
       <c r="AP57" s="32"/>
     </row>
     <row r="58" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="212" t="s">
+      <c r="A58" s="228" t="s">
         <v>127</v>
       </c>
       <c r="B58" s="141" t="s">
@@ -12445,7 +12457,7 @@
       <c r="AP58" s="26"/>
     </row>
     <row r="59" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="213"/>
+      <c r="A59" s="229"/>
       <c r="B59" s="142" t="s">
         <v>133</v>
       </c>
@@ -12491,7 +12503,7 @@
       <c r="AP59" s="32"/>
     </row>
     <row r="60" spans="1:51" s="40" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="212" t="s">
+      <c r="A60" s="228" t="s">
         <v>128</v>
       </c>
       <c r="B60" s="141" t="s">
@@ -12548,7 +12560,7 @@
       <c r="AY60" s="2"/>
     </row>
     <row r="61" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="226"/>
+      <c r="A61" s="240"/>
       <c r="B61" s="142" t="s">
         <v>133</v>
       </c>
@@ -12642,7 +12654,7 @@
       <c r="AP62" s="113"/>
     </row>
     <row r="63" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="223" t="s">
+      <c r="A63" s="237" t="s">
         <v>45</v>
       </c>
       <c r="B63" s="141" t="s">
@@ -12690,7 +12702,7 @@
       <c r="AP63" s="30"/>
     </row>
     <row r="64" spans="1:51" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A64" s="225"/>
+      <c r="A64" s="239"/>
       <c r="B64" s="142" t="s">
         <v>133</v>
       </c>
@@ -12736,7 +12748,7 @@
       <c r="AP64" s="30"/>
     </row>
     <row r="65" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A65" s="223" t="s">
+      <c r="A65" s="237" t="s">
         <v>46</v>
       </c>
       <c r="B65" s="141" t="s">
@@ -12784,7 +12796,7 @@
       <c r="AP65" s="24"/>
     </row>
     <row r="66" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="225"/>
+      <c r="A66" s="239"/>
       <c r="B66" s="142" t="s">
         <v>133</v>
       </c>
@@ -12830,7 +12842,7 @@
       <c r="AP66" s="32"/>
     </row>
     <row r="67" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="223" t="s">
+      <c r="A67" s="237" t="s">
         <v>120</v>
       </c>
       <c r="B67" s="141" t="s">
@@ -12878,7 +12890,7 @@
       <c r="AP67" s="24"/>
     </row>
     <row r="68" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="224"/>
+      <c r="A68" s="238"/>
       <c r="B68" s="142" t="s">
         <v>133</v>
       </c>
@@ -12965,14 +12977,14 @@
       <c r="AI69" s="101"/>
       <c r="AJ69" s="102"/>
       <c r="AK69" s="102"/>
-      <c r="AL69" s="102"/>
-      <c r="AM69" s="101"/>
-      <c r="AN69" s="102"/>
-      <c r="AO69" s="102"/>
-      <c r="AP69" s="102"/>
+      <c r="AL69" s="197"/>
+      <c r="AM69" s="100"/>
+      <c r="AN69" s="98"/>
+      <c r="AO69" s="98"/>
+      <c r="AP69" s="113"/>
     </row>
     <row r="70" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="258" t="s">
+      <c r="A70" s="192" t="s">
         <v>130</v>
       </c>
       <c r="B70" s="141" t="s">
@@ -13020,7 +13032,7 @@
       <c r="AP70" s="91"/>
     </row>
     <row r="71" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="259"/>
+      <c r="A71" s="193"/>
       <c r="B71" s="142" t="s">
         <v>133</v>
       </c>
@@ -13066,7 +13078,7 @@
       <c r="AP71" s="91"/>
     </row>
     <row r="72" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="258" t="s">
+      <c r="A72" s="192" t="s">
         <v>131</v>
       </c>
       <c r="B72" s="141" t="s">
@@ -13114,7 +13126,7 @@
       <c r="AP72" s="18"/>
     </row>
     <row r="73" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A73" s="259"/>
+      <c r="A73" s="193"/>
       <c r="B73" s="142" t="s">
         <v>133</v>
       </c>
@@ -13160,7 +13172,7 @@
       <c r="AP73" s="18"/>
     </row>
     <row r="74" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A74" s="258" t="s">
+      <c r="A74" s="192" t="s">
         <v>135</v>
       </c>
       <c r="B74" s="141" t="s">
@@ -13210,7 +13222,7 @@
       <c r="AP74" s="18"/>
     </row>
     <row r="75" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A75" s="259"/>
+      <c r="A75" s="193"/>
       <c r="B75" s="142" t="s">
         <v>133</v>
       </c>
@@ -13256,7 +13268,7 @@
       <c r="AP75" s="18"/>
     </row>
     <row r="76" spans="1:42" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A76" s="258" t="s">
+      <c r="A76" s="192" t="s">
         <v>136</v>
       </c>
       <c r="B76" s="141" t="s">
@@ -13299,7 +13311,7 @@
       <c r="AK76" s="155" t="s">
         <v>139</v>
       </c>
-      <c r="AL76" s="256" t="s">
+      <c r="AL76" s="190" t="s">
         <v>139</v>
       </c>
       <c r="AM76" s="23"/>
@@ -13308,7 +13320,7 @@
       <c r="AP76" s="18"/>
     </row>
     <row r="77" spans="1:42" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A77" s="259"/>
+      <c r="A77" s="193"/>
       <c r="B77" s="142" t="s">
         <v>133</v>
       </c>
@@ -13354,7 +13366,7 @@
       <c r="AP77" s="145"/>
     </row>
     <row r="78" spans="1:42" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A78" s="258" t="s">
+      <c r="A78" s="192" t="s">
         <v>137</v>
       </c>
       <c r="B78" s="141" t="s">
@@ -13395,7 +13407,7 @@
       <c r="AI78" s="27"/>
       <c r="AJ78" s="43"/>
       <c r="AK78" s="25"/>
-      <c r="AL78" s="257" t="s">
+      <c r="AL78" s="191" t="s">
         <v>139</v>
       </c>
       <c r="AM78" s="23"/>
@@ -13404,7 +13416,7 @@
       <c r="AP78" s="18"/>
     </row>
     <row r="79" spans="1:42" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A79" s="259"/>
+      <c r="A79" s="193"/>
       <c r="B79" s="142" t="s">
         <v>133</v>
       </c>
@@ -13450,11 +13462,11 @@
       <c r="AP79" s="44"/>
     </row>
     <row r="80" spans="1:42" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A80" s="250" t="s">
-        <v>166</v>
-      </c>
-      <c r="B80" s="168" t="s">
-        <v>143</v>
+      <c r="A80" s="184" t="s">
+        <v>159</v>
+      </c>
+      <c r="B80" s="196" t="s">
+        <v>146</v>
       </c>
       <c r="C80" s="96"/>
       <c r="D80" s="97"/>
@@ -13492,10 +13504,10 @@
       <c r="AJ80" s="97"/>
       <c r="AK80" s="98"/>
       <c r="AL80" s="99"/>
-      <c r="AM80" s="251"/>
-      <c r="AN80" s="252"/>
-      <c r="AO80" s="251"/>
-      <c r="AP80" s="253"/>
+      <c r="AM80" s="185"/>
+      <c r="AN80" s="186"/>
+      <c r="AO80" s="185"/>
+      <c r="AP80" s="187"/>
     </row>
   </sheetData>
   <mergeCells count="52">
@@ -13512,6 +13524,7 @@
     <mergeCell ref="AM3:AP3"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="E2:AP2"/>
+    <mergeCell ref="AE4:AH4"/>
     <mergeCell ref="AI4:AL4"/>
     <mergeCell ref="AM4:AP4"/>
     <mergeCell ref="C4:F4"/>
@@ -13519,21 +13532,22 @@
     <mergeCell ref="K4:N4"/>
     <mergeCell ref="O4:R4"/>
     <mergeCell ref="S4:V4"/>
+    <mergeCell ref="A56:A57"/>
     <mergeCell ref="A22:A23"/>
     <mergeCell ref="A20:A21"/>
     <mergeCell ref="W4:Z4"/>
     <mergeCell ref="AA4:AD4"/>
-    <mergeCell ref="AE4:AH4"/>
-    <mergeCell ref="A54:A55"/>
-    <mergeCell ref="A52:A53"/>
-    <mergeCell ref="A50:A51"/>
-    <mergeCell ref="A48:A49"/>
     <mergeCell ref="A67:A68"/>
     <mergeCell ref="A65:A66"/>
     <mergeCell ref="A63:A64"/>
     <mergeCell ref="A60:A61"/>
     <mergeCell ref="A58:A59"/>
-    <mergeCell ref="A56:A57"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="A54:A55"/>
+    <mergeCell ref="A52:A53"/>
+    <mergeCell ref="A50:A51"/>
+    <mergeCell ref="A48:A49"/>
+    <mergeCell ref="A24:A25"/>
     <mergeCell ref="A46:A47"/>
     <mergeCell ref="A44:A45"/>
     <mergeCell ref="A9:A10"/>
@@ -13549,8 +13563,6 @@
     <mergeCell ref="A11:A12"/>
     <mergeCell ref="A42:A43"/>
     <mergeCell ref="A28:A29"/>
-    <mergeCell ref="A26:A27"/>
-    <mergeCell ref="A24:A25"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.35" right="0.35" top="0.35" bottom="0.5" header="0.3" footer="0.3"/>
@@ -13574,49 +13586,49 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:59" ht="29.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="203" t="s">
+      <c r="A1" s="217" t="s">
         <v>93</v>
       </c>
-      <c r="B1" s="203"/>
-      <c r="C1" s="203"/>
-      <c r="D1" s="203"/>
-      <c r="E1" s="203"/>
-      <c r="F1" s="203"/>
-      <c r="G1" s="203"/>
-      <c r="H1" s="203"/>
-      <c r="I1" s="203"/>
-      <c r="J1" s="203"/>
-      <c r="K1" s="203"/>
-      <c r="L1" s="203"/>
-      <c r="M1" s="203"/>
-      <c r="N1" s="203"/>
-      <c r="O1" s="203"/>
-      <c r="P1" s="203"/>
-      <c r="Q1" s="203"/>
-      <c r="R1" s="203"/>
-      <c r="S1" s="203"/>
-      <c r="T1" s="203"/>
-      <c r="U1" s="203"/>
-      <c r="V1" s="203"/>
-      <c r="W1" s="203"/>
-      <c r="X1" s="203"/>
-      <c r="Y1" s="203"/>
-      <c r="Z1" s="203"/>
-      <c r="AA1" s="203"/>
-      <c r="AB1" s="203"/>
-      <c r="AC1" s="203"/>
-      <c r="AD1" s="203"/>
-      <c r="AE1" s="203"/>
-      <c r="AF1" s="203"/>
-      <c r="AG1" s="203"/>
-      <c r="AH1" s="203"/>
-      <c r="AI1" s="203"/>
-      <c r="AJ1" s="203"/>
-      <c r="AK1" s="203"/>
-      <c r="AL1" s="203"/>
-      <c r="AM1" s="203"/>
-      <c r="AN1" s="203"/>
-      <c r="AO1" s="203"/>
+      <c r="B1" s="217"/>
+      <c r="C1" s="217"/>
+      <c r="D1" s="217"/>
+      <c r="E1" s="217"/>
+      <c r="F1" s="217"/>
+      <c r="G1" s="217"/>
+      <c r="H1" s="217"/>
+      <c r="I1" s="217"/>
+      <c r="J1" s="217"/>
+      <c r="K1" s="217"/>
+      <c r="L1" s="217"/>
+      <c r="M1" s="217"/>
+      <c r="N1" s="217"/>
+      <c r="O1" s="217"/>
+      <c r="P1" s="217"/>
+      <c r="Q1" s="217"/>
+      <c r="R1" s="217"/>
+      <c r="S1" s="217"/>
+      <c r="T1" s="217"/>
+      <c r="U1" s="217"/>
+      <c r="V1" s="217"/>
+      <c r="W1" s="217"/>
+      <c r="X1" s="217"/>
+      <c r="Y1" s="217"/>
+      <c r="Z1" s="217"/>
+      <c r="AA1" s="217"/>
+      <c r="AB1" s="217"/>
+      <c r="AC1" s="217"/>
+      <c r="AD1" s="217"/>
+      <c r="AE1" s="217"/>
+      <c r="AF1" s="217"/>
+      <c r="AG1" s="217"/>
+      <c r="AH1" s="217"/>
+      <c r="AI1" s="217"/>
+      <c r="AJ1" s="217"/>
+      <c r="AK1" s="217"/>
+      <c r="AL1" s="217"/>
+      <c r="AM1" s="217"/>
+      <c r="AN1" s="217"/>
+      <c r="AO1" s="217"/>
     </row>
     <row r="2" spans="1:59" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="14" t="s">
@@ -13627,131 +13639,131 @@
       <c r="A3" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B3" s="208" t="s">
+      <c r="B3" s="222" t="s">
         <v>94</v>
       </c>
-      <c r="C3" s="209"/>
-      <c r="D3" s="209"/>
-      <c r="E3" s="210"/>
-      <c r="F3" s="208" t="s">
+      <c r="C3" s="223"/>
+      <c r="D3" s="223"/>
+      <c r="E3" s="224"/>
+      <c r="F3" s="222" t="s">
         <v>95</v>
       </c>
-      <c r="G3" s="209"/>
-      <c r="H3" s="209"/>
-      <c r="I3" s="210"/>
-      <c r="J3" s="208" t="s">
+      <c r="G3" s="223"/>
+      <c r="H3" s="223"/>
+      <c r="I3" s="224"/>
+      <c r="J3" s="222" t="s">
         <v>96</v>
       </c>
-      <c r="K3" s="209"/>
-      <c r="L3" s="209"/>
-      <c r="M3" s="210"/>
-      <c r="N3" s="208" t="s">
+      <c r="K3" s="223"/>
+      <c r="L3" s="223"/>
+      <c r="M3" s="224"/>
+      <c r="N3" s="222" t="s">
         <v>97</v>
       </c>
-      <c r="O3" s="209"/>
-      <c r="P3" s="209"/>
-      <c r="Q3" s="210"/>
-      <c r="R3" s="208" t="s">
+      <c r="O3" s="223"/>
+      <c r="P3" s="223"/>
+      <c r="Q3" s="224"/>
+      <c r="R3" s="222" t="s">
         <v>94</v>
       </c>
-      <c r="S3" s="209"/>
-      <c r="T3" s="209"/>
-      <c r="U3" s="210"/>
-      <c r="V3" s="208" t="s">
+      <c r="S3" s="223"/>
+      <c r="T3" s="223"/>
+      <c r="U3" s="224"/>
+      <c r="V3" s="222" t="s">
         <v>95</v>
       </c>
-      <c r="W3" s="209"/>
-      <c r="X3" s="209"/>
-      <c r="Y3" s="210"/>
-      <c r="Z3" s="208" t="s">
+      <c r="W3" s="223"/>
+      <c r="X3" s="223"/>
+      <c r="Y3" s="224"/>
+      <c r="Z3" s="222" t="s">
         <v>96</v>
       </c>
-      <c r="AA3" s="209"/>
-      <c r="AB3" s="209"/>
-      <c r="AC3" s="210"/>
-      <c r="AD3" s="208" t="s">
+      <c r="AA3" s="223"/>
+      <c r="AB3" s="223"/>
+      <c r="AC3" s="224"/>
+      <c r="AD3" s="222" t="s">
         <v>97</v>
       </c>
-      <c r="AE3" s="209"/>
-      <c r="AF3" s="209"/>
-      <c r="AG3" s="210"/>
-      <c r="AH3" s="208" t="s">
+      <c r="AE3" s="223"/>
+      <c r="AF3" s="223"/>
+      <c r="AG3" s="224"/>
+      <c r="AH3" s="222" t="s">
         <v>98</v>
       </c>
-      <c r="AI3" s="209"/>
-      <c r="AJ3" s="209"/>
-      <c r="AK3" s="210"/>
-      <c r="AL3" s="208" t="s">
+      <c r="AI3" s="223"/>
+      <c r="AJ3" s="223"/>
+      <c r="AK3" s="224"/>
+      <c r="AL3" s="222" t="s">
         <v>94</v>
       </c>
-      <c r="AM3" s="209"/>
-      <c r="AN3" s="209"/>
-      <c r="AO3" s="210"/>
+      <c r="AM3" s="223"/>
+      <c r="AN3" s="223"/>
+      <c r="AO3" s="224"/>
     </row>
     <row r="4" spans="1:59" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="20">
         <v>46139</v>
       </c>
-      <c r="B4" s="205" t="s">
+      <c r="B4" s="219" t="s">
         <v>99</v>
       </c>
-      <c r="C4" s="206"/>
-      <c r="D4" s="206"/>
-      <c r="E4" s="207"/>
-      <c r="F4" s="205" t="s">
+      <c r="C4" s="220"/>
+      <c r="D4" s="220"/>
+      <c r="E4" s="221"/>
+      <c r="F4" s="219" t="s">
         <v>100</v>
       </c>
-      <c r="G4" s="206"/>
-      <c r="H4" s="206"/>
-      <c r="I4" s="207"/>
-      <c r="J4" s="205" t="s">
+      <c r="G4" s="220"/>
+      <c r="H4" s="220"/>
+      <c r="I4" s="221"/>
+      <c r="J4" s="219" t="s">
         <v>101</v>
       </c>
-      <c r="K4" s="206"/>
-      <c r="L4" s="206"/>
-      <c r="M4" s="207"/>
-      <c r="N4" s="205" t="s">
+      <c r="K4" s="220"/>
+      <c r="L4" s="220"/>
+      <c r="M4" s="221"/>
+      <c r="N4" s="219" t="s">
         <v>102</v>
       </c>
-      <c r="O4" s="206"/>
-      <c r="P4" s="206"/>
-      <c r="Q4" s="207"/>
-      <c r="R4" s="205" t="s">
+      <c r="O4" s="220"/>
+      <c r="P4" s="220"/>
+      <c r="Q4" s="221"/>
+      <c r="R4" s="219" t="s">
         <v>103</v>
       </c>
-      <c r="S4" s="206"/>
-      <c r="T4" s="206"/>
-      <c r="U4" s="207"/>
-      <c r="V4" s="205" t="s">
+      <c r="S4" s="220"/>
+      <c r="T4" s="220"/>
+      <c r="U4" s="221"/>
+      <c r="V4" s="219" t="s">
         <v>104</v>
       </c>
-      <c r="W4" s="206"/>
-      <c r="X4" s="206"/>
-      <c r="Y4" s="207"/>
-      <c r="Z4" s="205" t="s">
+      <c r="W4" s="220"/>
+      <c r="X4" s="220"/>
+      <c r="Y4" s="221"/>
+      <c r="Z4" s="219" t="s">
         <v>105</v>
       </c>
-      <c r="AA4" s="206"/>
-      <c r="AB4" s="206"/>
-      <c r="AC4" s="207"/>
-      <c r="AD4" s="205" t="s">
+      <c r="AA4" s="220"/>
+      <c r="AB4" s="220"/>
+      <c r="AC4" s="221"/>
+      <c r="AD4" s="219" t="s">
         <v>106</v>
       </c>
-      <c r="AE4" s="206"/>
-      <c r="AF4" s="206"/>
-      <c r="AG4" s="207"/>
-      <c r="AH4" s="205" t="s">
+      <c r="AE4" s="220"/>
+      <c r="AF4" s="220"/>
+      <c r="AG4" s="221"/>
+      <c r="AH4" s="219" t="s">
         <v>107</v>
       </c>
-      <c r="AI4" s="206"/>
-      <c r="AJ4" s="206"/>
-      <c r="AK4" s="207"/>
-      <c r="AL4" s="205" t="s">
+      <c r="AI4" s="220"/>
+      <c r="AJ4" s="220"/>
+      <c r="AK4" s="221"/>
+      <c r="AL4" s="219" t="s">
         <v>108</v>
       </c>
-      <c r="AM4" s="206"/>
-      <c r="AN4" s="206"/>
-      <c r="AO4" s="207"/>
+      <c r="AM4" s="220"/>
+      <c r="AN4" s="220"/>
+      <c r="AO4" s="221"/>
     </row>
     <row r="5" spans="1:59" s="38" customFormat="1" ht="33" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="123" t="s">
@@ -15315,38 +15327,38 @@
       </c>
     </row>
     <row r="40" spans="1:41" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="Z40" s="230" t="s">
+      <c r="Z40" s="244" t="s">
         <v>21</v>
       </c>
-      <c r="AA40" s="231"/>
-      <c r="AB40" s="234" t="s">
+      <c r="AA40" s="245"/>
+      <c r="AB40" s="248" t="s">
         <v>88</v>
       </c>
-      <c r="AC40" s="235"/>
-      <c r="AD40" s="238" t="s">
+      <c r="AC40" s="249"/>
+      <c r="AD40" s="252" t="s">
         <v>22</v>
       </c>
-      <c r="AE40" s="239"/>
-      <c r="AF40" s="242" t="s">
+      <c r="AE40" s="253"/>
+      <c r="AF40" s="256" t="s">
         <v>50</v>
       </c>
-      <c r="AG40" s="243"/>
-      <c r="AH40" s="246" t="s">
+      <c r="AG40" s="257"/>
+      <c r="AH40" s="260" t="s">
         <v>49</v>
       </c>
-      <c r="AI40" s="247"/>
+      <c r="AI40" s="261"/>
     </row>
     <row r="41" spans="1:41" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="Z41" s="232"/>
-      <c r="AA41" s="233"/>
-      <c r="AB41" s="236"/>
-      <c r="AC41" s="237"/>
-      <c r="AD41" s="240"/>
-      <c r="AE41" s="241"/>
-      <c r="AF41" s="244"/>
-      <c r="AG41" s="245"/>
-      <c r="AH41" s="248"/>
-      <c r="AI41" s="249"/>
+      <c r="Z41" s="246"/>
+      <c r="AA41" s="247"/>
+      <c r="AB41" s="250"/>
+      <c r="AC41" s="251"/>
+      <c r="AD41" s="254"/>
+      <c r="AE41" s="255"/>
+      <c r="AF41" s="258"/>
+      <c r="AG41" s="259"/>
+      <c r="AH41" s="262"/>
+      <c r="AI41" s="263"/>
     </row>
   </sheetData>
   <mergeCells count="26">

</xml_diff>